<commit_message>
Catch up - small changes
Small changes that have accrued over last month, preparing to proceed w/ updates and improvements.
</commit_message>
<xml_diff>
--- a/data/templates/financial_template_v2_2026.xlsx
+++ b/data/templates/financial_template_v2_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfizer-my.sharepoint.com/personal/hoveyo_pfizer_com/Documents/financial-automation-project/data/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="171" documentId="8_{783183DD-73AE-4283-AD85-EEFD805851D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67E8D884-7862-41E5-98D0-4F52412DF91E}"/>
+  <xr:revisionPtr revIDLastSave="186" documentId="8_{783183DD-73AE-4283-AD85-EEFD805851D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2275B3F8-8E5A-4910-A117-4523E2FD9255}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="12480" tabRatio="590" xr2:uid="{0996C49B-04E6-42AE-AA83-2F64BE89A626}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Template" sheetId="5" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template!$A$14:$BY$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template!$A$15:$BY$15</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -1613,7 +1613,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1822,6 +1822,15 @@
     <xf numFmtId="3" fontId="3" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1834,14 +1843,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1850,7 +1853,35 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{EFDA3BDD-7E2C-4F3B-BEB7-091BB23895D4}"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="7">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF7C80"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF7C80"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2182,7 +2213,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{177F1DEB-197D-49C6-A2E3-152C1AC7B373}">
-  <dimension ref="A1:EI66"/>
+  <dimension ref="A1:EI67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -2202,137 +2233,151 @@
     <col min="76" max="76" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:139" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="1" spans="1:139" x14ac:dyDescent="0.25">
+      <c r="A1" s="13"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+    </row>
     <row r="2" spans="1:139" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
+      <c r="A2" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="34">
+        <v>2026</v>
+      </c>
+      <c r="F2" s="34"/>
+      <c r="G2" s="35">
+        <f>C2</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
     </row>
     <row r="3" spans="1:139" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="34" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="33">
+        <v>0</v>
+      </c>
+      <c r="D3" s="34">
+        <v>2321511</v>
       </c>
       <c r="E3" s="34">
         <v>2026</v>
       </c>
       <c r="F3" s="34"/>
       <c r="G3" s="35">
-        <f>C3</f>
         <v>0</v>
       </c>
       <c r="H3" s="46"/>
       <c r="I3" s="46"/>
       <c r="J3" s="46"/>
-      <c r="S3" s="1"/>
-      <c r="T3" s="1"/>
-      <c r="U3" s="1"/>
     </row>
     <row r="4" spans="1:139" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="33">
-        <v>0</v>
-      </c>
-      <c r="D4" s="34">
-        <v>2321511</v>
-      </c>
-      <c r="E4" s="34">
-        <v>2026</v>
-      </c>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35">
-        <v>0</v>
-      </c>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46"/>
+      <c r="A4" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="30"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
     </row>
     <row r="5" spans="1:139" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="30"/>
+        <v>5</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>6</v>
+      </c>
       <c r="C5" s="37"/>
       <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="47"/>
-      <c r="J5" s="47"/>
-    </row>
-    <row r="6" spans="1:139" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="39" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="40" t="str">
+      <c r="E5" s="40" t="str">
         <f>IF(SUMIFS(BV:BV,A:A,"Contingency")&gt;0,"Contingency is "&amp;TEXT(SUMIFS(BV:BV,A:A,"Contingency"),"$#,##"),IF(SUMIFS(BV:BV,A:A,"Contingency")&lt;0,"Overspent by "&amp;TEXT(SUMIFS(BV:BV,A:A,"Contingency"),"$#,##"),"No contingency"))</f>
         <v>No contingency</v>
       </c>
-      <c r="F6" s="40"/>
-      <c r="G6" s="17"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+    </row>
+    <row r="6" spans="1:139" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="18"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22"/>
       <c r="H6" s="37"/>
       <c r="I6" s="37"/>
       <c r="J6" s="37"/>
-      <c r="K6" s="42"/>
-      <c r="L6" s="6"/>
     </row>
     <row r="7" spans="1:139" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="37"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="6"/>
     </row>
-    <row r="8" spans="1:139" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:139" x14ac:dyDescent="0.25">
+      <c r="A8" s="105" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="106"/>
+      <c r="D8" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+    </row>
     <row r="9" spans="1:139" x14ac:dyDescent="0.25">
-      <c r="A9" s="105" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="106"/>
-      <c r="D9" s="55" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="43"/>
+      <c r="A9" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:139" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="25" t="s">
-        <v>9</v>
+    <row r="10" spans="1:139" x14ac:dyDescent="0.25">
+      <c r="A10" s="26" t="s">
+        <v>12</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>10</v>
@@ -2344,16 +2389,13 @@
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
       <c r="J10" s="12"/>
-      <c r="K10" s="44"/>
-      <c r="BW10" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="K10" s="43"/>
     </row>
-    <row r="11" spans="1:139" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="23" t="s">
+    <row r="11" spans="1:139" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="24" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="11"/>
@@ -2364,137 +2406,18 @@
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
       <c r="K11" s="44"/>
-      <c r="L11" s="110" t="s">
+      <c r="BW11" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:139" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K12" s="44"/>
+      <c r="L12" s="113" t="s">
         <v>13</v>
       </c>
-      <c r="M11" s="111"/>
-      <c r="N11" s="107" cm="1">
-        <f t="array" ref="N11">SUM(Q15:Q65)+SUM(_xlfn._xlws.FILTER(P15:P65,Q15:Q65=""))+SUM(_xlfn._xlws.FILTER(O15:O65,(P15:P65="")*(Q15:Q65="")))+SUMIFS(R15:R65,Q15:Q65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(N15:N65)</f>
-        <v>0</v>
-      </c>
-      <c r="O11" s="108"/>
-      <c r="P11" s="108"/>
-      <c r="Q11" s="108"/>
-      <c r="R11" s="109"/>
-      <c r="S11" s="107" cm="1">
-        <f t="array" ref="S11">SUM(V15:V65)+SUM(_xlfn._xlws.FILTER(U15:U65,V15:V65=""))+SUM(_xlfn._xlws.FILTER(T15:T65,(U15:U65="")*(V15:V65="")))+SUMIFS(W15:W65,V15:V65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(S15:S65)</f>
-        <v>0</v>
-      </c>
-      <c r="T11" s="108"/>
-      <c r="U11" s="108"/>
-      <c r="V11" s="108"/>
-      <c r="W11" s="109"/>
-      <c r="X11" s="107" cm="1">
-        <f t="array" ref="X11">SUM(AA15:AA65)+SUM(_xlfn._xlws.FILTER(Z15:Z65,AA15:AA65=""))+SUM(_xlfn._xlws.FILTER(Y15:Y65,(Z15:Z65="")*(AA15:AA65="")))+SUMIFS(AB15:AB65,AA15:AA65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(X15:X65)</f>
-        <v>0</v>
-      </c>
-      <c r="Y11" s="108"/>
-      <c r="Z11" s="108"/>
-      <c r="AA11" s="108"/>
-      <c r="AB11" s="109"/>
-      <c r="AC11" s="107" cm="1">
-        <f t="array" ref="AC11">SUM(AF15:AF65)+SUM(_xlfn._xlws.FILTER(AE15:AE65,AF15:AF65=""))+SUM(_xlfn._xlws.FILTER(AD15:AD65,(AE15:AE65="")*(AF15:AF65="")))+SUMIFS(AG15:AG65,AF15:AF65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(AC15:AC65)</f>
-        <v>0</v>
-      </c>
-      <c r="AD11" s="108"/>
-      <c r="AE11" s="108"/>
-      <c r="AF11" s="108"/>
-      <c r="AG11" s="109"/>
-      <c r="AH11" s="107" cm="1">
-        <f t="array" ref="AH11">SUM(AK15:AK65)+SUM(_xlfn._xlws.FILTER(AJ15:AJ65,AK15:AK65=""))+SUM(_xlfn._xlws.FILTER(AI15:AI65,(AJ15:AJ65="")*(AK15:AK65="")))+SUMIFS(AL15:AL65,AK15:AK65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(AH15:AH65)</f>
-        <v>0</v>
-      </c>
-      <c r="AI11" s="108"/>
-      <c r="AJ11" s="108"/>
-      <c r="AK11" s="108"/>
-      <c r="AL11" s="109"/>
-      <c r="AM11" s="107" cm="1">
-        <f t="array" ref="AM11">SUM(AP15:AP65)+SUM(_xlfn._xlws.FILTER(AO15:AO65,AP15:AP65=""))+SUM(_xlfn._xlws.FILTER(AN15:AN65,(AO15:AO65="")*(AP15:AP65="")))+SUMIFS(AQ15:AQ65,AP15:AP65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(AM15:AM65)</f>
-        <v>0</v>
-      </c>
-      <c r="AN11" s="108"/>
-      <c r="AO11" s="108"/>
-      <c r="AP11" s="108"/>
-      <c r="AQ11" s="109"/>
-      <c r="AR11" s="107" cm="1">
-        <f t="array" ref="AR11">SUM(AU15:AU65)+SUM(_xlfn._xlws.FILTER(AT15:AT65,AU15:AU65=""))+SUM(_xlfn._xlws.FILTER(AS15:AS65,(AT15:AT65="")*(AU15:AU65="")))+SUMIFS(AV15:AV65,AU15:AU65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(AR15:AR65)</f>
-        <v>0</v>
-      </c>
-      <c r="AS11" s="108"/>
-      <c r="AT11" s="108"/>
-      <c r="AU11" s="108"/>
-      <c r="AV11" s="109"/>
-      <c r="AW11" s="107" cm="1">
-        <f t="array" ref="AW11">SUM(AZ15:AZ65)+SUM(_xlfn._xlws.FILTER(AY15:AY65,AZ15:AZ65=""))+SUM(_xlfn._xlws.FILTER(AX15:AX65,(AY15:AY65="")*(AZ15:AZ65="")))+SUMIFS(BA15:BA65,AZ15:AZ65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(AW15:AW65)</f>
-        <v>0</v>
-      </c>
-      <c r="AX11" s="108"/>
-      <c r="AY11" s="108"/>
-      <c r="AZ11" s="108"/>
-      <c r="BA11" s="109"/>
-      <c r="BB11" s="107" cm="1">
-        <f t="array" ref="BB11">SUM(BE15:BE65)+SUM(_xlfn._xlws.FILTER(BD15:BD65,BE15:BE65=""))+SUM(_xlfn._xlws.FILTER(BC15:BC65,(BD15:BD65="")*(BE15:BE65="")))+SUMIFS(BF15:BF65,BE15:BE65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(BB15:BB65)</f>
-        <v>0</v>
-      </c>
-      <c r="BC11" s="108"/>
-      <c r="BD11" s="108"/>
-      <c r="BE11" s="108"/>
-      <c r="BF11" s="109"/>
-      <c r="BG11" s="107" cm="1">
-        <f t="array" ref="BG11">SUM(BJ15:BJ65)+SUM(_xlfn._xlws.FILTER(BI15:BI65,BJ15:BJ65=""))+SUM(_xlfn._xlws.FILTER(BH15:BH65,(BI15:BI65="")*(BJ15:BJ65="")))+SUMIFS(BK15:BK65,BJ15:BJ65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(BG15:BG65)</f>
-        <v>0</v>
-      </c>
-      <c r="BH11" s="108"/>
-      <c r="BI11" s="108"/>
-      <c r="BJ11" s="108"/>
-      <c r="BK11" s="109"/>
-      <c r="BL11" s="107" cm="1">
-        <f t="array" ref="BL11">SUM(BO15:BO65)+SUM(_xlfn._xlws.FILTER(BN15:BN65,BO15:BO65=""))+SUM(_xlfn._xlws.FILTER(BM15:BM65,(BN15:BN65="")*(BO15:BO65="")))+SUMIFS(BP15:BP65,BO15:BO65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(BL15:BL65)</f>
-        <v>0</v>
-      </c>
-      <c r="BM11" s="108"/>
-      <c r="BN11" s="108"/>
-      <c r="BO11" s="108"/>
-      <c r="BP11" s="109"/>
-      <c r="BQ11" s="107" cm="1">
-        <f t="array" ref="BQ11">SUM(BT15:BT65)+SUM(_xlfn._xlws.FILTER(BS15:BS65,BT15:BT65=""))+SUM(_xlfn._xlws.FILTER(BR15:BR65,(BS15:BS65="")*(BT15:BT65="")))+SUMIFS(BU15:BU65,BT15:BT65,"&lt;&gt;"&amp;"",$P$15:$P$65,"&lt;&gt;"&amp;"")+SUM(BQ15:BQ65)</f>
-        <v>0</v>
-      </c>
-      <c r="BR11" s="108"/>
-      <c r="BS11" s="108"/>
-      <c r="BT11" s="108"/>
-      <c r="BU11" s="109"/>
-      <c r="BV11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="BW11" s="5">
-        <f>BW13-BV13</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:139" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="45" t="s">
-        <v>16</v>
-      </c>
-      <c r="L12" s="112" t="s">
-        <v>17</v>
-      </c>
-      <c r="M12" s="113"/>
+      <c r="M12" s="114"/>
       <c r="N12" s="107" cm="1">
-        <f t="array" ref="N12">SUM(Q15:Q65)+SUM(_xlfn._xlws.FILTER(P15:P65,Q15:Q65=""))+SUM(_xlfn._xlws.FILTER(O15:O65,(P15:P65="")*(Q15:Q65="")))</f>
+        <f t="array" ref="N12">SUM(Q16:Q66)+SUM(_xlfn._xlws.FILTER(P16:P66,Q16:Q66=""))+SUM(_xlfn._xlws.FILTER(O16:O66,(P16:P66="")*(Q16:Q66="")))+SUMIFS(R16:R66,Q16:Q66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(N16:N66)</f>
         <v>0</v>
       </c>
       <c r="O12" s="108"/>
@@ -2502,7 +2425,7 @@
       <c r="Q12" s="108"/>
       <c r="R12" s="109"/>
       <c r="S12" s="107" cm="1">
-        <f t="array" ref="S12">SUM(V15:V65)+SUM(_xlfn._xlws.FILTER(U15:U65,V15:V65=""))+SUM(_xlfn._xlws.FILTER(T15:T65,(U15:U65="")*(V15:V65="")))</f>
+        <f t="array" ref="S12">SUM(V16:V66)+SUM(_xlfn._xlws.FILTER(U16:U66,V16:V66=""))+SUM(_xlfn._xlws.FILTER(T16:T66,(U16:U66="")*(V16:V66="")))+SUMIFS(W16:W66,V16:V66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(S16:S66)</f>
         <v>0</v>
       </c>
       <c r="T12" s="108"/>
@@ -2510,7 +2433,7 @@
       <c r="V12" s="108"/>
       <c r="W12" s="109"/>
       <c r="X12" s="107" cm="1">
-        <f t="array" ref="X12">SUM(AA15:AA65)+SUM(_xlfn._xlws.FILTER(Z15:Z65,AA15:AA65=""))+SUM(_xlfn._xlws.FILTER(Y15:Y65,(Z15:Z65="")*(AA15:AA65="")))</f>
+        <f t="array" ref="X12">SUM(AA16:AA66)+SUM(_xlfn._xlws.FILTER(Z16:Z66,AA16:AA66=""))+SUM(_xlfn._xlws.FILTER(Y16:Y66,(Z16:Z66="")*(AA16:AA66="")))+SUMIFS(AB16:AB66,AA16:AA66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(X16:X66)</f>
         <v>0</v>
       </c>
       <c r="Y12" s="108"/>
@@ -2518,7 +2441,7 @@
       <c r="AA12" s="108"/>
       <c r="AB12" s="109"/>
       <c r="AC12" s="107" cm="1">
-        <f t="array" ref="AC12">SUM(AF15:AF65)+SUM(_xlfn._xlws.FILTER(AE15:AE65,AF15:AF65=""))+SUM(_xlfn._xlws.FILTER(AD15:AD65,(AE15:AE65="")*(AF15:AF65="")))</f>
+        <f t="array" ref="AC12">SUM(AF16:AF66)+SUM(_xlfn._xlws.FILTER(AE16:AE66,AF16:AF66=""))+SUM(_xlfn._xlws.FILTER(AD16:AD66,(AE16:AE66="")*(AF16:AF66="")))+SUMIFS(AG16:AG66,AF16:AF66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(AC16:AC66)</f>
         <v>0</v>
       </c>
       <c r="AD12" s="108"/>
@@ -2526,7 +2449,7 @@
       <c r="AF12" s="108"/>
       <c r="AG12" s="109"/>
       <c r="AH12" s="107" cm="1">
-        <f t="array" ref="AH12">SUM(AK15:AK65)+SUM(_xlfn._xlws.FILTER(AJ15:AJ65,AK15:AK65=""))+SUM(_xlfn._xlws.FILTER(AI15:AI65,(AJ15:AJ65="")*(AK15:AK65="")))</f>
+        <f t="array" ref="AH12">SUM(AK16:AK66)+SUM(_xlfn._xlws.FILTER(AJ16:AJ66,AK16:AK66=""))+SUM(_xlfn._xlws.FILTER(AI16:AI66,(AJ16:AJ66="")*(AK16:AK66="")))+SUMIFS(AL16:AL66,AK16:AK66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(AH16:AH66)</f>
         <v>0</v>
       </c>
       <c r="AI12" s="108"/>
@@ -2534,7 +2457,7 @@
       <c r="AK12" s="108"/>
       <c r="AL12" s="109"/>
       <c r="AM12" s="107" cm="1">
-        <f t="array" ref="AM12">SUM(AP15:AP65)+SUM(_xlfn._xlws.FILTER(AO15:AO65,AP15:AP65=""))+SUM(_xlfn._xlws.FILTER(AN15:AN65,(AO15:AO65="")*(AP15:AP65="")))</f>
+        <f t="array" ref="AM12">SUM(AP16:AP66)+SUM(_xlfn._xlws.FILTER(AO16:AO66,AP16:AP66=""))+SUM(_xlfn._xlws.FILTER(AN16:AN66,(AO16:AO66="")*(AP16:AP66="")))+SUMIFS(AQ16:AQ66,AP16:AP66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(AM16:AM66)</f>
         <v>0</v>
       </c>
       <c r="AN12" s="108"/>
@@ -2542,7 +2465,7 @@
       <c r="AP12" s="108"/>
       <c r="AQ12" s="109"/>
       <c r="AR12" s="107" cm="1">
-        <f t="array" ref="AR12">SUM(AU15:AU65)+SUM(_xlfn._xlws.FILTER(AT15:AT65,AU15:AU65=""))+SUM(_xlfn._xlws.FILTER(AS15:AS65,(AT15:AT65="")*(AU15:AU65="")))</f>
+        <f t="array" ref="AR12">SUM(AU16:AU66)+SUM(_xlfn._xlws.FILTER(AT16:AT66,AU16:AU66=""))+SUM(_xlfn._xlws.FILTER(AS16:AS66,(AT16:AT66="")*(AU16:AU66="")))+SUMIFS(AV16:AV66,AU16:AU66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(AR16:AR66)</f>
         <v>0</v>
       </c>
       <c r="AS12" s="108"/>
@@ -2550,7 +2473,7 @@
       <c r="AU12" s="108"/>
       <c r="AV12" s="109"/>
       <c r="AW12" s="107" cm="1">
-        <f t="array" ref="AW12">SUM(AZ15:AZ65)+SUM(_xlfn._xlws.FILTER(AY15:AY65,AZ15:AZ65=""))+SUM(_xlfn._xlws.FILTER(AX15:AX65,(AY15:AY65="")*(AZ15:AZ65="")))</f>
+        <f t="array" ref="AW12">SUM(AZ16:AZ66)+SUM(_xlfn._xlws.FILTER(AY16:AY66,AZ16:AZ66=""))+SUM(_xlfn._xlws.FILTER(AX16:AX66,(AY16:AY66="")*(AZ16:AZ66="")))+SUMIFS(BA16:BA66,AZ16:AZ66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(AW16:AW66)</f>
         <v>0</v>
       </c>
       <c r="AX12" s="108"/>
@@ -2558,7 +2481,7 @@
       <c r="AZ12" s="108"/>
       <c r="BA12" s="109"/>
       <c r="BB12" s="107" cm="1">
-        <f t="array" ref="BB12">SUM(BE15:BE65)+SUM(_xlfn._xlws.FILTER(BD15:BD65,BE15:BE65=""))+SUM(_xlfn._xlws.FILTER(BC15:BC65,(BD15:BD65="")*(BE15:BE65="")))</f>
+        <f t="array" ref="BB12">SUM(BE16:BE66)+SUM(_xlfn._xlws.FILTER(BD16:BD66,BE16:BE66=""))+SUM(_xlfn._xlws.FILTER(BC16:BC66,(BD16:BD66="")*(BE16:BE66="")))+SUMIFS(BF16:BF66,BE16:BE66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(BB16:BB66)</f>
         <v>0</v>
       </c>
       <c r="BC12" s="108"/>
@@ -2566,7 +2489,7 @@
       <c r="BE12" s="108"/>
       <c r="BF12" s="109"/>
       <c r="BG12" s="107" cm="1">
-        <f t="array" ref="BG12">SUM(BJ15:BJ65)+SUM(_xlfn._xlws.FILTER(BI15:BI65,BJ15:BJ65=""))+SUM(_xlfn._xlws.FILTER(BH15:BH65,(BI15:BI65="")*(BJ15:BJ65="")))</f>
+        <f t="array" ref="BG12">SUM(BJ16:BJ66)+SUM(_xlfn._xlws.FILTER(BI16:BI66,BJ16:BJ66=""))+SUM(_xlfn._xlws.FILTER(BH16:BH66,(BI16:BI66="")*(BJ16:BJ66="")))+SUMIFS(BK16:BK66,BJ16:BJ66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(BG16:BG66)</f>
         <v>0</v>
       </c>
       <c r="BH12" s="108"/>
@@ -2574,7 +2497,7 @@
       <c r="BJ12" s="108"/>
       <c r="BK12" s="109"/>
       <c r="BL12" s="107" cm="1">
-        <f t="array" ref="BL12">SUM(BO15:BO65)+SUM(_xlfn._xlws.FILTER(BN15:BN65,BO15:BO65=""))+SUM(_xlfn._xlws.FILTER(BM15:BM65,(BN15:BN65="")*(BO15:BO65="")))</f>
+        <f t="array" ref="BL12">SUM(BO16:BO66)+SUM(_xlfn._xlws.FILTER(BN16:BN66,BO16:BO66=""))+SUM(_xlfn._xlws.FILTER(BM16:BM66,(BN16:BN66="")*(BO16:BO66="")))+SUMIFS(BP16:BP66,BO16:BO66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(BL16:BL66)</f>
         <v>0</v>
       </c>
       <c r="BM12" s="108"/>
@@ -2582,617 +2505,524 @@
       <c r="BO12" s="108"/>
       <c r="BP12" s="109"/>
       <c r="BQ12" s="107" cm="1">
-        <f t="array" ref="BQ12">SUM(BT15:BT65)+SUM(_xlfn._xlws.FILTER(BS15:BS65,BT15:BT65=""))+SUM(_xlfn._xlws.FILTER(BR15:BR65,(BS15:BS65="")*(BT15:BT65="")))</f>
+        <f t="array" ref="BQ12">SUM(BT16:BT66)+SUM(_xlfn._xlws.FILTER(BS16:BS66,BT16:BT66=""))+SUM(_xlfn._xlws.FILTER(BR16:BR66,(BS16:BS66="")*(BT16:BT66="")))+SUMIFS(BU16:BU66,BT16:BT66,"&lt;&gt;"&amp;"",$P$16:$P$66,"&lt;&gt;"&amp;"")+SUM(BQ16:BQ66)</f>
         <v>0</v>
       </c>
       <c r="BR12" s="108"/>
       <c r="BS12" s="108"/>
       <c r="BT12" s="108"/>
       <c r="BU12" s="109"/>
-      <c r="BV12" s="4"/>
-      <c r="BW12" s="5"/>
+      <c r="BV12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="BW12" s="5">
+        <f>BW14-BV14</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:139" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
+    <row r="13" spans="1:139" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K13" s="45" t="s">
+        <v>16</v>
+      </c>
+      <c r="L13" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="M13" s="116"/>
+      <c r="N13" s="107" cm="1">
+        <f t="array" ref="N13">SUM(Q16:Q66)+SUM(_xlfn._xlws.FILTER(P16:P66,Q16:Q66=""))+SUM(_xlfn._xlws.FILTER(O16:O66,(P16:P66="")*(Q16:Q66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="O13" s="108"/>
+      <c r="P13" s="108"/>
+      <c r="Q13" s="108"/>
+      <c r="R13" s="109"/>
+      <c r="S13" s="107" cm="1">
+        <f t="array" ref="S13">SUM(V16:V66)+SUM(_xlfn._xlws.FILTER(U16:U66,V16:V66=""))+SUM(_xlfn._xlws.FILTER(T16:T66,(U16:U66="")*(V16:V66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="T13" s="108"/>
+      <c r="U13" s="108"/>
+      <c r="V13" s="108"/>
+      <c r="W13" s="109"/>
+      <c r="X13" s="107" cm="1">
+        <f t="array" ref="X13">SUM(AA16:AA66)+SUM(_xlfn._xlws.FILTER(Z16:Z66,AA16:AA66=""))+SUM(_xlfn._xlws.FILTER(Y16:Y66,(Z16:Z66="")*(AA16:AA66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="Y13" s="108"/>
+      <c r="Z13" s="108"/>
+      <c r="AA13" s="108"/>
+      <c r="AB13" s="109"/>
+      <c r="AC13" s="107" cm="1">
+        <f t="array" ref="AC13">SUM(AF16:AF66)+SUM(_xlfn._xlws.FILTER(AE16:AE66,AF16:AF66=""))+SUM(_xlfn._xlws.FILTER(AD16:AD66,(AE16:AE66="")*(AF16:AF66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="AD13" s="108"/>
+      <c r="AE13" s="108"/>
+      <c r="AF13" s="108"/>
+      <c r="AG13" s="109"/>
+      <c r="AH13" s="107" cm="1">
+        <f t="array" ref="AH13">SUM(AK16:AK66)+SUM(_xlfn._xlws.FILTER(AJ16:AJ66,AK16:AK66=""))+SUM(_xlfn._xlws.FILTER(AI16:AI66,(AJ16:AJ66="")*(AK16:AK66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="AI13" s="108"/>
+      <c r="AJ13" s="108"/>
+      <c r="AK13" s="108"/>
+      <c r="AL13" s="109"/>
+      <c r="AM13" s="107" cm="1">
+        <f t="array" ref="AM13">SUM(AP16:AP66)+SUM(_xlfn._xlws.FILTER(AO16:AO66,AP16:AP66=""))+SUM(_xlfn._xlws.FILTER(AN16:AN66,(AO16:AO66="")*(AP16:AP66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="AN13" s="108"/>
+      <c r="AO13" s="108"/>
+      <c r="AP13" s="108"/>
+      <c r="AQ13" s="109"/>
+      <c r="AR13" s="107" cm="1">
+        <f t="array" ref="AR13">SUM(AU16:AU66)+SUM(_xlfn._xlws.FILTER(AT16:AT66,AU16:AU66=""))+SUM(_xlfn._xlws.FILTER(AS16:AS66,(AT16:AT66="")*(AU16:AU66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="AS13" s="108"/>
+      <c r="AT13" s="108"/>
+      <c r="AU13" s="108"/>
+      <c r="AV13" s="109"/>
+      <c r="AW13" s="107" cm="1">
+        <f t="array" ref="AW13">SUM(AZ16:AZ66)+SUM(_xlfn._xlws.FILTER(AY16:AY66,AZ16:AZ66=""))+SUM(_xlfn._xlws.FILTER(AX16:AX66,(AY16:AY66="")*(AZ16:AZ66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="AX13" s="108"/>
+      <c r="AY13" s="108"/>
+      <c r="AZ13" s="108"/>
+      <c r="BA13" s="109"/>
+      <c r="BB13" s="107" cm="1">
+        <f t="array" ref="BB13">SUM(BE16:BE66)+SUM(_xlfn._xlws.FILTER(BD16:BD66,BE16:BE66=""))+SUM(_xlfn._xlws.FILTER(BC16:BC66,(BD16:BD66="")*(BE16:BE66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="BC13" s="108"/>
+      <c r="BD13" s="108"/>
+      <c r="BE13" s="108"/>
+      <c r="BF13" s="109"/>
+      <c r="BG13" s="107" cm="1">
+        <f t="array" ref="BG13">SUM(BJ16:BJ66)+SUM(_xlfn._xlws.FILTER(BI16:BI66,BJ16:BJ66=""))+SUM(_xlfn._xlws.FILTER(BH16:BH66,(BI16:BI66="")*(BJ16:BJ66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="BH13" s="108"/>
+      <c r="BI13" s="108"/>
+      <c r="BJ13" s="108"/>
+      <c r="BK13" s="109"/>
+      <c r="BL13" s="107" cm="1">
+        <f t="array" ref="BL13">SUM(BO16:BO66)+SUM(_xlfn._xlws.FILTER(BN16:BN66,BO16:BO66=""))+SUM(_xlfn._xlws.FILTER(BM16:BM66,(BN16:BN66="")*(BO16:BO66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="BM13" s="108"/>
+      <c r="BN13" s="108"/>
+      <c r="BO13" s="108"/>
+      <c r="BP13" s="109"/>
+      <c r="BQ13" s="107" cm="1">
+        <f t="array" ref="BQ13">SUM(BT16:BT66)+SUM(_xlfn._xlws.FILTER(BS16:BS66,BT16:BT66=""))+SUM(_xlfn._xlws.FILTER(BR16:BR66,(BS16:BS66="")*(BT16:BT66="")))</f>
+        <v>0</v>
+      </c>
+      <c r="BR13" s="108"/>
+      <c r="BS13" s="108"/>
+      <c r="BT13" s="108"/>
+      <c r="BU13" s="109"/>
+      <c r="BV13" s="4"/>
+      <c r="BW13" s="5"/>
+    </row>
+    <row r="14" spans="1:139" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="54">
-        <f>SUBTOTAL(9,K15:K16)</f>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="54">
+        <f>SUBTOTAL(9,K16:K17)</f>
         <v>190781</v>
       </c>
-      <c r="L13" s="112" t="s">
+      <c r="L14" s="115" t="s">
         <v>19</v>
       </c>
-      <c r="M13" s="113"/>
-      <c r="N13" s="114">
+      <c r="M14" s="116"/>
+      <c r="N14" s="110">
         <v>46053</v>
       </c>
-      <c r="O13" s="115" t="s">
+      <c r="O14" s="111" t="s">
         <v>20</v>
       </c>
-      <c r="P13" s="115"/>
-      <c r="Q13" s="115"/>
-      <c r="R13" s="115"/>
-      <c r="S13" s="114">
+      <c r="P14" s="111"/>
+      <c r="Q14" s="111"/>
+      <c r="R14" s="111"/>
+      <c r="S14" s="110">
         <v>46054</v>
       </c>
-      <c r="T13" s="115"/>
-      <c r="U13" s="115"/>
-      <c r="V13" s="115"/>
-      <c r="W13" s="116"/>
-      <c r="X13" s="114">
+      <c r="T14" s="111"/>
+      <c r="U14" s="111"/>
+      <c r="V14" s="111"/>
+      <c r="W14" s="112"/>
+      <c r="X14" s="110">
         <v>46112</v>
       </c>
-      <c r="Y13" s="115" t="s">
+      <c r="Y14" s="111" t="s">
         <v>21</v>
       </c>
-      <c r="Z13" s="115"/>
-      <c r="AA13" s="115"/>
-      <c r="AB13" s="116"/>
-      <c r="AC13" s="114">
+      <c r="Z14" s="111"/>
+      <c r="AA14" s="111"/>
+      <c r="AB14" s="112"/>
+      <c r="AC14" s="110">
         <v>46142</v>
       </c>
-      <c r="AD13" s="115" t="s">
+      <c r="AD14" s="111" t="s">
         <v>22</v>
       </c>
-      <c r="AE13" s="115"/>
-      <c r="AF13" s="115"/>
-      <c r="AG13" s="116"/>
-      <c r="AH13" s="114">
+      <c r="AE14" s="111"/>
+      <c r="AF14" s="111"/>
+      <c r="AG14" s="112"/>
+      <c r="AH14" s="110">
         <v>46173</v>
       </c>
-      <c r="AI13" s="115" t="s">
+      <c r="AI14" s="111" t="s">
         <v>23</v>
       </c>
-      <c r="AJ13" s="115"/>
-      <c r="AK13" s="115"/>
-      <c r="AL13" s="116"/>
-      <c r="AM13" s="114">
+      <c r="AJ14" s="111"/>
+      <c r="AK14" s="111"/>
+      <c r="AL14" s="112"/>
+      <c r="AM14" s="110">
         <v>46203</v>
       </c>
-      <c r="AN13" s="115" t="s">
+      <c r="AN14" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="AO13" s="115"/>
-      <c r="AP13" s="115"/>
-      <c r="AQ13" s="116"/>
-      <c r="AR13" s="114">
+      <c r="AO14" s="111"/>
+      <c r="AP14" s="111"/>
+      <c r="AQ14" s="112"/>
+      <c r="AR14" s="110">
         <v>46234</v>
       </c>
-      <c r="AS13" s="115" t="s">
+      <c r="AS14" s="111" t="s">
         <v>25</v>
       </c>
-      <c r="AT13" s="115"/>
-      <c r="AU13" s="115"/>
-      <c r="AV13" s="116"/>
-      <c r="AW13" s="114">
+      <c r="AT14" s="111"/>
+      <c r="AU14" s="111"/>
+      <c r="AV14" s="112"/>
+      <c r="AW14" s="110">
         <v>46265</v>
       </c>
-      <c r="AX13" s="115" t="s">
+      <c r="AX14" s="111" t="s">
         <v>26</v>
       </c>
-      <c r="AY13" s="115"/>
-      <c r="AZ13" s="115"/>
-      <c r="BA13" s="116"/>
-      <c r="BB13" s="114">
+      <c r="AY14" s="111"/>
+      <c r="AZ14" s="111"/>
+      <c r="BA14" s="112"/>
+      <c r="BB14" s="110">
         <v>46295</v>
       </c>
-      <c r="BC13" s="115" t="s">
+      <c r="BC14" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="BD13" s="115"/>
-      <c r="BE13" s="115"/>
-      <c r="BF13" s="116"/>
-      <c r="BG13" s="114">
+      <c r="BD14" s="111"/>
+      <c r="BE14" s="111"/>
+      <c r="BF14" s="112"/>
+      <c r="BG14" s="110">
         <v>46326</v>
       </c>
-      <c r="BH13" s="115" t="s">
+      <c r="BH14" s="111" t="s">
         <v>28</v>
       </c>
-      <c r="BI13" s="115"/>
-      <c r="BJ13" s="115"/>
-      <c r="BK13" s="116"/>
-      <c r="BL13" s="114">
+      <c r="BI14" s="111"/>
+      <c r="BJ14" s="111"/>
+      <c r="BK14" s="112"/>
+      <c r="BL14" s="110">
         <v>46356</v>
       </c>
-      <c r="BM13" s="115" t="s">
+      <c r="BM14" s="111" t="s">
         <v>29</v>
       </c>
-      <c r="BN13" s="115"/>
-      <c r="BO13" s="115"/>
-      <c r="BP13" s="116"/>
-      <c r="BQ13" s="114">
+      <c r="BN14" s="111"/>
+      <c r="BO14" s="111"/>
+      <c r="BP14" s="112"/>
+      <c r="BQ14" s="110">
         <v>46387</v>
       </c>
-      <c r="BR13" s="115" t="s">
+      <c r="BR14" s="111" t="s">
         <v>30</v>
       </c>
-      <c r="BS13" s="115"/>
-      <c r="BT13" s="115"/>
-      <c r="BU13" s="116"/>
-      <c r="BV13" s="7">
-        <f>SUM(BV15:BV65)</f>
-        <v>0</v>
-      </c>
-      <c r="BW13" s="8"/>
-      <c r="BY13" s="3"/>
+      <c r="BS14" s="111"/>
+      <c r="BT14" s="111"/>
+      <c r="BU14" s="112"/>
+      <c r="BV14" s="7">
+        <f>SUM(BV16:BV66)</f>
+        <v>0</v>
+      </c>
+      <c r="BW14" s="8"/>
+      <c r="BY14" s="3"/>
     </row>
-    <row r="14" spans="1:139" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="56" t="s">
+    <row r="15" spans="1:139" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="57" t="s">
+      <c r="B15" s="57" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="58" t="s">
+      <c r="C15" s="58" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="59" t="s">
+      <c r="D15" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="60" t="s">
+      <c r="E15" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="F14" s="60" t="s">
+      <c r="F15" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="58" t="s">
+      <c r="G15" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="H14" s="58" t="s">
+      <c r="H15" s="58" t="s">
         <v>38</v>
       </c>
-      <c r="I14" s="58" t="s">
+      <c r="I15" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="J14" s="58" t="s">
+      <c r="J15" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="K14" s="61" t="s">
+      <c r="K15" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="L14" s="62" t="s">
+      <c r="L15" s="62" t="s">
         <v>41</v>
       </c>
-      <c r="M14" s="48" t="s">
+      <c r="M15" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="N14" s="51" t="s">
+      <c r="N15" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="O14" s="52" t="s">
+      <c r="O15" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="P14" s="52" t="s">
+      <c r="P15" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="Q14" s="52" t="s">
+      <c r="Q15" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="R14" s="50" t="s">
+      <c r="R15" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="S14" s="63" t="s">
+      <c r="S15" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="T14" s="52" t="s">
+      <c r="T15" s="52" t="s">
         <v>49</v>
       </c>
-      <c r="U14" s="52" t="s">
+      <c r="U15" s="52" t="s">
         <v>50</v>
       </c>
-      <c r="V14" s="64" t="s">
+      <c r="V15" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="W14" s="65" t="s">
+      <c r="W15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="X14" s="63" t="s">
+      <c r="X15" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="Y14" s="52" t="s">
+      <c r="Y15" s="52" t="s">
         <v>53</v>
       </c>
-      <c r="Z14" s="52" t="s">
+      <c r="Z15" s="52" t="s">
         <v>54</v>
       </c>
-      <c r="AA14" s="64" t="s">
+      <c r="AA15" s="64" t="s">
         <v>55</v>
       </c>
-      <c r="AB14" s="65" t="s">
+      <c r="AB15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="AC14" s="63" t="s">
+      <c r="AC15" s="63" t="s">
         <v>56</v>
       </c>
-      <c r="AD14" s="52" t="s">
+      <c r="AD15" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="AE14" s="52" t="s">
+      <c r="AE15" s="52" t="s">
         <v>58</v>
       </c>
-      <c r="AF14" s="64" t="s">
+      <c r="AF15" s="64" t="s">
         <v>59</v>
       </c>
-      <c r="AG14" s="65" t="s">
+      <c r="AG15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="AH14" s="63" t="s">
+      <c r="AH15" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="AI14" s="52" t="s">
+      <c r="AI15" s="52" t="s">
         <v>61</v>
       </c>
-      <c r="AJ14" s="52" t="s">
+      <c r="AJ15" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="AK14" s="64" t="s">
+      <c r="AK15" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="AL14" s="65" t="s">
+      <c r="AL15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="AM14" s="63" t="s">
+      <c r="AM15" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="AN14" s="52" t="s">
+      <c r="AN15" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="AO14" s="52" t="s">
+      <c r="AO15" s="52" t="s">
         <v>66</v>
       </c>
-      <c r="AP14" s="64" t="s">
+      <c r="AP15" s="64" t="s">
         <v>67</v>
       </c>
-      <c r="AQ14" s="65" t="s">
+      <c r="AQ15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="AR14" s="63" t="s">
+      <c r="AR15" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="AS14" s="52" t="s">
+      <c r="AS15" s="52" t="s">
         <v>69</v>
       </c>
-      <c r="AT14" s="52" t="s">
+      <c r="AT15" s="52" t="s">
         <v>70</v>
       </c>
-      <c r="AU14" s="64" t="s">
+      <c r="AU15" s="64" t="s">
         <v>71</v>
       </c>
-      <c r="AV14" s="65" t="s">
+      <c r="AV15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="AW14" s="63" t="s">
+      <c r="AW15" s="63" t="s">
         <v>72</v>
       </c>
-      <c r="AX14" s="52" t="s">
+      <c r="AX15" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="AY14" s="52" t="s">
+      <c r="AY15" s="52" t="s">
         <v>74</v>
       </c>
-      <c r="AZ14" s="64" t="s">
+      <c r="AZ15" s="64" t="s">
         <v>75</v>
       </c>
-      <c r="BA14" s="65" t="s">
+      <c r="BA15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="BB14" s="63" t="s">
+      <c r="BB15" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="BC14" s="52" t="s">
+      <c r="BC15" s="52" t="s">
         <v>77</v>
       </c>
-      <c r="BD14" s="52" t="s">
+      <c r="BD15" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="BE14" s="64" t="s">
+      <c r="BE15" s="64" t="s">
         <v>79</v>
       </c>
-      <c r="BF14" s="65" t="s">
+      <c r="BF15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="BG14" s="63" t="s">
+      <c r="BG15" s="63" t="s">
         <v>80</v>
       </c>
-      <c r="BH14" s="52" t="s">
+      <c r="BH15" s="52" t="s">
         <v>81</v>
       </c>
-      <c r="BI14" s="52" t="s">
+      <c r="BI15" s="52" t="s">
         <v>82</v>
       </c>
-      <c r="BJ14" s="64" t="s">
+      <c r="BJ15" s="64" t="s">
         <v>83</v>
       </c>
-      <c r="BK14" s="65" t="s">
+      <c r="BK15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="BL14" s="63" t="s">
+      <c r="BL15" s="63" t="s">
         <v>84</v>
       </c>
-      <c r="BM14" s="52" t="s">
+      <c r="BM15" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="BN14" s="52" t="s">
+      <c r="BN15" s="52" t="s">
         <v>86</v>
       </c>
-      <c r="BO14" s="64" t="s">
+      <c r="BO15" s="64" t="s">
         <v>87</v>
       </c>
-      <c r="BP14" s="65" t="s">
+      <c r="BP15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="BQ14" s="63" t="s">
+      <c r="BQ15" s="63" t="s">
         <v>88</v>
       </c>
-      <c r="BR14" s="52" t="s">
+      <c r="BR15" s="52" t="s">
         <v>89</v>
       </c>
-      <c r="BS14" s="52" t="s">
+      <c r="BS15" s="52" t="s">
         <v>90</v>
       </c>
-      <c r="BT14" s="64" t="s">
+      <c r="BT15" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="BU14" s="65" t="s">
+      <c r="BU15" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="BV14" s="51" t="s">
+      <c r="BV15" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="BW14" s="52" t="s">
+      <c r="BW15" s="52" t="s">
         <v>93</v>
       </c>
-      <c r="BX14" s="48" t="s">
+      <c r="BX15" s="48" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="15" spans="1:139" x14ac:dyDescent="0.25">
-      <c r="A15" s="79" t="s">
-        <v>97</v>
-      </c>
-      <c r="B15" s="94">
-        <v>9501133449</v>
-      </c>
-      <c r="C15" s="96">
-        <v>45993</v>
-      </c>
-      <c r="D15" s="96">
-        <v>46173</v>
-      </c>
-      <c r="E15" s="81" t="s">
-        <v>98</v>
-      </c>
-      <c r="F15" s="80" t="s">
-        <v>99</v>
-      </c>
-      <c r="G15" s="80">
-        <v>41500000</v>
-      </c>
-      <c r="H15" s="80">
-        <v>3840</v>
-      </c>
-      <c r="I15" s="80" t="s">
-        <v>100</v>
-      </c>
-      <c r="J15" s="80">
-        <v>2430238</v>
-      </c>
-      <c r="K15" s="97">
-        <v>66363</v>
-      </c>
-      <c r="L15" s="100" t="s">
-        <v>165</v>
-      </c>
-      <c r="M15" s="101" t="s">
-        <v>166</v>
-      </c>
-      <c r="N15" s="82"/>
-      <c r="O15" s="83"/>
-      <c r="P15" s="83"/>
-      <c r="Q15" s="84"/>
-      <c r="R15" s="84">
-        <f>P15-Q15</f>
-        <v>0</v>
-      </c>
-      <c r="S15" s="85"/>
-      <c r="T15" s="83"/>
-      <c r="U15" s="83"/>
-      <c r="V15" s="84"/>
-      <c r="W15" s="86">
-        <f>U15-V15</f>
-        <v>0</v>
-      </c>
-      <c r="X15" s="87"/>
-      <c r="Y15" s="83"/>
-      <c r="Z15" s="83"/>
-      <c r="AA15" s="84"/>
-      <c r="AB15" s="86">
-        <f>Z15-AA15</f>
-        <v>0</v>
-      </c>
-      <c r="AC15" s="87"/>
-      <c r="AD15" s="83"/>
-      <c r="AE15" s="83"/>
-      <c r="AF15" s="83"/>
-      <c r="AG15" s="86">
-        <f>AE15-AF15</f>
-        <v>0</v>
-      </c>
-      <c r="AH15" s="87"/>
-      <c r="AI15" s="83"/>
-      <c r="AJ15" s="83"/>
-      <c r="AK15" s="83"/>
-      <c r="AL15" s="86">
-        <f>AJ15-AK15</f>
-        <v>0</v>
-      </c>
-      <c r="AM15" s="87"/>
-      <c r="AN15" s="83"/>
-      <c r="AO15" s="83"/>
-      <c r="AP15" s="83"/>
-      <c r="AQ15" s="86">
-        <f>AO15-AP15</f>
-        <v>0</v>
-      </c>
-      <c r="AR15" s="87"/>
-      <c r="AS15" s="83"/>
-      <c r="AT15" s="83"/>
-      <c r="AU15" s="83"/>
-      <c r="AV15" s="86">
-        <f>AT15-AU15</f>
-        <v>0</v>
-      </c>
-      <c r="AW15" s="87"/>
-      <c r="AX15" s="83"/>
-      <c r="AY15" s="83"/>
-      <c r="AZ15" s="83"/>
-      <c r="BA15" s="86">
-        <f>AY15-AZ15</f>
-        <v>0</v>
-      </c>
-      <c r="BB15" s="87"/>
-      <c r="BC15" s="83"/>
-      <c r="BD15" s="83"/>
-      <c r="BE15" s="83"/>
-      <c r="BF15" s="86">
-        <f>BD15-BE15</f>
-        <v>0</v>
-      </c>
-      <c r="BG15" s="87"/>
-      <c r="BH15" s="83"/>
-      <c r="BI15" s="83"/>
-      <c r="BJ15" s="83"/>
-      <c r="BK15" s="86">
-        <f>BI15-BJ15</f>
-        <v>0</v>
-      </c>
-      <c r="BL15" s="87"/>
-      <c r="BM15" s="83"/>
-      <c r="BN15" s="83"/>
-      <c r="BO15" s="83"/>
-      <c r="BP15" s="86">
-        <f>BN15-BO15</f>
-        <v>0</v>
-      </c>
-      <c r="BQ15" s="87"/>
-      <c r="BR15" s="83"/>
-      <c r="BS15" s="83"/>
-      <c r="BT15" s="83"/>
-      <c r="BU15" s="86">
-        <f>BS15-BT15</f>
-        <v>0</v>
-      </c>
-      <c r="BV15" s="88">
-        <v>0</v>
-      </c>
-      <c r="BW15" s="89"/>
-      <c r="BX15" s="90"/>
-      <c r="BY15" s="78"/>
-      <c r="BZ15" s="78"/>
-      <c r="CA15" s="78"/>
-      <c r="CB15" s="78"/>
-      <c r="CC15" s="78"/>
-      <c r="CD15" s="78"/>
-      <c r="CE15" s="78"/>
-      <c r="CF15" s="78"/>
-      <c r="CG15" s="78"/>
-      <c r="CH15" s="78"/>
-      <c r="CI15" s="78"/>
-      <c r="CJ15" s="78"/>
-      <c r="CK15" s="78"/>
-      <c r="CL15" s="78"/>
-      <c r="CM15" s="78"/>
-      <c r="CN15" s="78"/>
-      <c r="CO15" s="78"/>
-      <c r="CP15" s="78"/>
-      <c r="CQ15" s="78"/>
-      <c r="CR15" s="78"/>
-      <c r="CS15" s="78"/>
-      <c r="CT15" s="78"/>
-      <c r="CU15" s="78"/>
-      <c r="CV15" s="78"/>
-      <c r="CW15" s="78"/>
-      <c r="CX15" s="78"/>
-      <c r="CY15" s="78"/>
-      <c r="CZ15" s="78"/>
-      <c r="DA15" s="78"/>
-      <c r="DB15" s="78"/>
-      <c r="DC15" s="78"/>
-      <c r="DD15" s="78"/>
-      <c r="DE15" s="78"/>
-      <c r="DF15" s="78"/>
-      <c r="DG15" s="78"/>
-      <c r="DH15" s="78"/>
-      <c r="DI15" s="78"/>
-      <c r="DJ15" s="78"/>
-      <c r="DK15" s="78"/>
-      <c r="DL15" s="78"/>
-      <c r="DM15" s="78"/>
-      <c r="DN15" s="78"/>
-      <c r="DO15" s="78"/>
-      <c r="DP15" s="78"/>
-      <c r="DQ15" s="78"/>
-      <c r="DR15" s="78"/>
-      <c r="DS15" s="78"/>
-      <c r="DT15" s="78"/>
-      <c r="DU15" s="78"/>
-      <c r="DV15" s="78"/>
-      <c r="DW15" s="78"/>
-      <c r="DX15" s="78"/>
-      <c r="DY15" s="78"/>
-      <c r="DZ15" s="78"/>
-      <c r="EA15" s="78"/>
-      <c r="EB15" s="78"/>
-      <c r="EC15" s="78"/>
-      <c r="ED15" s="78"/>
-      <c r="EE15" s="78"/>
-      <c r="EF15" s="78"/>
-      <c r="EG15" s="78"/>
-      <c r="EH15" s="78"/>
-      <c r="EI15" s="78"/>
     </row>
     <row r="16" spans="1:139" x14ac:dyDescent="0.25">
-      <c r="A16" s="91" t="s">
+      <c r="A16" s="79" t="s">
         <v>97</v>
       </c>
-      <c r="B16" s="83">
-        <v>9501133442</v>
-      </c>
-      <c r="C16" s="98">
+      <c r="B16" s="94">
+        <v>9501133449</v>
+      </c>
+      <c r="C16" s="96">
         <v>45993</v>
       </c>
-      <c r="D16" s="98">
-        <v>46356</v>
-      </c>
-      <c r="E16" s="92" t="s">
-        <v>101</v>
-      </c>
-      <c r="F16" s="92" t="s">
-        <v>102</v>
-      </c>
-      <c r="G16" s="92">
+      <c r="D16" s="96">
+        <v>46173</v>
+      </c>
+      <c r="E16" s="81" t="s">
+        <v>98</v>
+      </c>
+      <c r="F16" s="80" t="s">
+        <v>99</v>
+      </c>
+      <c r="G16" s="80">
         <v>41500000</v>
       </c>
-      <c r="H16" s="92">
+      <c r="H16" s="80">
         <v>3840</v>
       </c>
-      <c r="I16" s="92" t="s">
+      <c r="I16" s="80" t="s">
         <v>100</v>
       </c>
-      <c r="J16" s="92">
+      <c r="J16" s="80">
         <v>2430238</v>
       </c>
-      <c r="K16" s="99">
-        <v>124418</v>
-      </c>
-      <c r="L16" s="102" t="s">
-        <v>167</v>
-      </c>
-      <c r="M16" s="103" t="s">
+      <c r="K16" s="97">
+        <v>66363</v>
+      </c>
+      <c r="L16" s="100" t="s">
+        <v>165</v>
+      </c>
+      <c r="M16" s="101" t="s">
         <v>166</v>
       </c>
       <c r="N16" s="82"/>
@@ -3222,7 +3052,7 @@
       <c r="AC16" s="87"/>
       <c r="AD16" s="83"/>
       <c r="AE16" s="83"/>
-      <c r="AF16" s="84"/>
+      <c r="AF16" s="83"/>
       <c r="AG16" s="86">
         <f>AE16-AF16</f>
         <v>0</v>
@@ -3230,7 +3060,7 @@
       <c r="AH16" s="87"/>
       <c r="AI16" s="83"/>
       <c r="AJ16" s="83"/>
-      <c r="AK16" s="84"/>
+      <c r="AK16" s="83"/>
       <c r="AL16" s="86">
         <f>AJ16-AK16</f>
         <v>0</v>
@@ -3238,7 +3068,7 @@
       <c r="AM16" s="87"/>
       <c r="AN16" s="83"/>
       <c r="AO16" s="83"/>
-      <c r="AP16" s="84"/>
+      <c r="AP16" s="83"/>
       <c r="AQ16" s="86">
         <f>AO16-AP16</f>
         <v>0</v>
@@ -3246,7 +3076,7 @@
       <c r="AR16" s="87"/>
       <c r="AS16" s="83"/>
       <c r="AT16" s="83"/>
-      <c r="AU16" s="84"/>
+      <c r="AU16" s="83"/>
       <c r="AV16" s="86">
         <f>AT16-AU16</f>
         <v>0</v>
@@ -3254,7 +3084,7 @@
       <c r="AW16" s="87"/>
       <c r="AX16" s="83"/>
       <c r="AY16" s="83"/>
-      <c r="AZ16" s="84"/>
+      <c r="AZ16" s="83"/>
       <c r="BA16" s="86">
         <f>AY16-AZ16</f>
         <v>0</v>
@@ -3262,7 +3092,7 @@
       <c r="BB16" s="87"/>
       <c r="BC16" s="83"/>
       <c r="BD16" s="83"/>
-      <c r="BE16" s="84"/>
+      <c r="BE16" s="83"/>
       <c r="BF16" s="86">
         <f>BD16-BE16</f>
         <v>0</v>
@@ -3270,7 +3100,7 @@
       <c r="BG16" s="87"/>
       <c r="BH16" s="83"/>
       <c r="BI16" s="83"/>
-      <c r="BJ16" s="84"/>
+      <c r="BJ16" s="83"/>
       <c r="BK16" s="86">
         <f>BI16-BJ16</f>
         <v>0</v>
@@ -3278,7 +3108,7 @@
       <c r="BL16" s="87"/>
       <c r="BM16" s="83"/>
       <c r="BN16" s="83"/>
-      <c r="BO16" s="84"/>
+      <c r="BO16" s="83"/>
       <c r="BP16" s="86">
         <f>BN16-BO16</f>
         <v>0</v>
@@ -3286,12 +3116,12 @@
       <c r="BQ16" s="87"/>
       <c r="BR16" s="83"/>
       <c r="BS16" s="83"/>
-      <c r="BT16" s="84"/>
+      <c r="BT16" s="83"/>
       <c r="BU16" s="86">
         <f>BS16-BT16</f>
         <v>0</v>
       </c>
-      <c r="BV16" s="85">
+      <c r="BV16" s="88">
         <v>0</v>
       </c>
       <c r="BW16" s="89"/>
@@ -3360,42 +3190,42 @@
       <c r="EH16" s="78"/>
       <c r="EI16" s="78"/>
     </row>
-    <row r="17" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:139" x14ac:dyDescent="0.25">
       <c r="A17" s="91" t="s">
         <v>97</v>
       </c>
       <c r="B17" s="83">
-        <v>9100561560</v>
+        <v>9501133442</v>
       </c>
       <c r="C17" s="98">
-        <v>46137</v>
+        <v>45993</v>
       </c>
       <c r="D17" s="98">
-        <v>46501</v>
+        <v>46356</v>
       </c>
       <c r="E17" s="92" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F17" s="92" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G17" s="92">
-        <v>61010000</v>
+        <v>41500000</v>
       </c>
       <c r="H17" s="92">
-        <v>1400</v>
+        <v>3840</v>
       </c>
       <c r="I17" s="92" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="J17" s="92">
-        <v>2321403</v>
+        <v>2430238</v>
       </c>
       <c r="K17" s="99">
-        <v>21098.22</v>
-      </c>
-      <c r="L17" s="104" t="s">
-        <v>168</v>
+        <v>124418</v>
+      </c>
+      <c r="L17" s="102" t="s">
+        <v>167</v>
       </c>
       <c r="M17" s="103" t="s">
         <v>166</v>
@@ -3405,7 +3235,7 @@
       <c r="P17" s="83"/>
       <c r="Q17" s="84"/>
       <c r="R17" s="84">
-        <f t="shared" ref="R17:R24" si="0">P17-Q17</f>
+        <f>P17-Q17</f>
         <v>0</v>
       </c>
       <c r="S17" s="85"/>
@@ -3413,7 +3243,7 @@
       <c r="U17" s="83"/>
       <c r="V17" s="84"/>
       <c r="W17" s="86">
-        <f t="shared" ref="W17:W24" si="1">U17-V17</f>
+        <f>U17-V17</f>
         <v>0</v>
       </c>
       <c r="X17" s="87"/>
@@ -3421,7 +3251,7 @@
       <c r="Z17" s="83"/>
       <c r="AA17" s="84"/>
       <c r="AB17" s="86">
-        <f t="shared" ref="AB17:AB24" si="2">Z17-AA17</f>
+        <f>Z17-AA17</f>
         <v>0</v>
       </c>
       <c r="AC17" s="87"/>
@@ -3429,7 +3259,7 @@
       <c r="AE17" s="83"/>
       <c r="AF17" s="84"/>
       <c r="AG17" s="86">
-        <f t="shared" ref="AG17:AG24" si="3">AE17-AF17</f>
+        <f>AE17-AF17</f>
         <v>0</v>
       </c>
       <c r="AH17" s="87"/>
@@ -3437,7 +3267,7 @@
       <c r="AJ17" s="83"/>
       <c r="AK17" s="84"/>
       <c r="AL17" s="86">
-        <f t="shared" ref="AL17:AL24" si="4">AJ17-AK17</f>
+        <f>AJ17-AK17</f>
         <v>0</v>
       </c>
       <c r="AM17" s="87"/>
@@ -3445,7 +3275,7 @@
       <c r="AO17" s="83"/>
       <c r="AP17" s="84"/>
       <c r="AQ17" s="86">
-        <f t="shared" ref="AQ17:AQ24" si="5">AO17-AP17</f>
+        <f>AO17-AP17</f>
         <v>0</v>
       </c>
       <c r="AR17" s="87"/>
@@ -3453,7 +3283,7 @@
       <c r="AT17" s="83"/>
       <c r="AU17" s="84"/>
       <c r="AV17" s="86">
-        <f t="shared" ref="AV17:AV24" si="6">AT17-AU17</f>
+        <f>AT17-AU17</f>
         <v>0</v>
       </c>
       <c r="AW17" s="87"/>
@@ -3461,7 +3291,7 @@
       <c r="AY17" s="83"/>
       <c r="AZ17" s="84"/>
       <c r="BA17" s="86">
-        <f t="shared" ref="BA17:BA24" si="7">AY17-AZ17</f>
+        <f>AY17-AZ17</f>
         <v>0</v>
       </c>
       <c r="BB17" s="87"/>
@@ -3469,7 +3299,7 @@
       <c r="BD17" s="83"/>
       <c r="BE17" s="84"/>
       <c r="BF17" s="86">
-        <f t="shared" ref="BF17:BF24" si="8">BD17-BE17</f>
+        <f>BD17-BE17</f>
         <v>0</v>
       </c>
       <c r="BG17" s="87"/>
@@ -3477,7 +3307,7 @@
       <c r="BI17" s="83"/>
       <c r="BJ17" s="84"/>
       <c r="BK17" s="86">
-        <f t="shared" ref="BK17:BK24" si="9">BI17-BJ17</f>
+        <f>BI17-BJ17</f>
         <v>0</v>
       </c>
       <c r="BL17" s="87"/>
@@ -3485,7 +3315,7 @@
       <c r="BN17" s="83"/>
       <c r="BO17" s="84"/>
       <c r="BP17" s="86">
-        <f t="shared" ref="BP17:BP24" si="10">BN17-BO17</f>
+        <f>BN17-BO17</f>
         <v>0</v>
       </c>
       <c r="BQ17" s="87"/>
@@ -3493,7 +3323,7 @@
       <c r="BS17" s="83"/>
       <c r="BT17" s="84"/>
       <c r="BU17" s="86">
-        <f t="shared" ref="BU17:BU24" si="11">BS17-BT17</f>
+        <f>BS17-BT17</f>
         <v>0</v>
       </c>
       <c r="BV17" s="85">
@@ -3501,37 +3331,116 @@
       </c>
       <c r="BW17" s="89"/>
       <c r="BX17" s="90"/>
+      <c r="BY17" s="78"/>
+      <c r="BZ17" s="78"/>
+      <c r="CA17" s="78"/>
+      <c r="CB17" s="78"/>
+      <c r="CC17" s="78"/>
+      <c r="CD17" s="78"/>
+      <c r="CE17" s="78"/>
+      <c r="CF17" s="78"/>
+      <c r="CG17" s="78"/>
+      <c r="CH17" s="78"/>
+      <c r="CI17" s="78"/>
+      <c r="CJ17" s="78"/>
+      <c r="CK17" s="78"/>
+      <c r="CL17" s="78"/>
+      <c r="CM17" s="78"/>
+      <c r="CN17" s="78"/>
+      <c r="CO17" s="78"/>
+      <c r="CP17" s="78"/>
+      <c r="CQ17" s="78"/>
+      <c r="CR17" s="78"/>
+      <c r="CS17" s="78"/>
+      <c r="CT17" s="78"/>
+      <c r="CU17" s="78"/>
+      <c r="CV17" s="78"/>
+      <c r="CW17" s="78"/>
+      <c r="CX17" s="78"/>
+      <c r="CY17" s="78"/>
+      <c r="CZ17" s="78"/>
+      <c r="DA17" s="78"/>
+      <c r="DB17" s="78"/>
+      <c r="DC17" s="78"/>
+      <c r="DD17" s="78"/>
+      <c r="DE17" s="78"/>
+      <c r="DF17" s="78"/>
+      <c r="DG17" s="78"/>
+      <c r="DH17" s="78"/>
+      <c r="DI17" s="78"/>
+      <c r="DJ17" s="78"/>
+      <c r="DK17" s="78"/>
+      <c r="DL17" s="78"/>
+      <c r="DM17" s="78"/>
+      <c r="DN17" s="78"/>
+      <c r="DO17" s="78"/>
+      <c r="DP17" s="78"/>
+      <c r="DQ17" s="78"/>
+      <c r="DR17" s="78"/>
+      <c r="DS17" s="78"/>
+      <c r="DT17" s="78"/>
+      <c r="DU17" s="78"/>
+      <c r="DV17" s="78"/>
+      <c r="DW17" s="78"/>
+      <c r="DX17" s="78"/>
+      <c r="DY17" s="78"/>
+      <c r="DZ17" s="78"/>
+      <c r="EA17" s="78"/>
+      <c r="EB17" s="78"/>
+      <c r="EC17" s="78"/>
+      <c r="ED17" s="78"/>
+      <c r="EE17" s="78"/>
+      <c r="EF17" s="78"/>
+      <c r="EG17" s="78"/>
+      <c r="EH17" s="78"/>
+      <c r="EI17" s="78"/>
     </row>
-    <row r="18" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:139" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="91" t="s">
         <v>97</v>
       </c>
       <c r="B18" s="83">
-        <v>9501079958</v>
+        <v>9100561560</v>
       </c>
       <c r="C18" s="98">
-        <v>45931</v>
+        <v>46137</v>
       </c>
       <c r="D18" s="98">
-        <v>46265</v>
+        <v>46501</v>
       </c>
       <c r="E18" s="92" t="s">
-        <v>106</v>
-      </c>
-      <c r="F18" s="92"/>
-      <c r="G18" s="92"/>
-      <c r="H18" s="92"/>
-      <c r="I18" s="92"/>
-      <c r="J18" s="92"/>
-      <c r="K18" s="93"/>
-      <c r="L18" s="104"/>
-      <c r="M18" s="103"/>
+        <v>103</v>
+      </c>
+      <c r="F18" s="92" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18" s="92">
+        <v>61010000</v>
+      </c>
+      <c r="H18" s="92">
+        <v>1400</v>
+      </c>
+      <c r="I18" s="92" t="s">
+        <v>105</v>
+      </c>
+      <c r="J18" s="92">
+        <v>2321403</v>
+      </c>
+      <c r="K18" s="99">
+        <v>21098.22</v>
+      </c>
+      <c r="L18" s="104" t="s">
+        <v>168</v>
+      </c>
+      <c r="M18" s="103" t="s">
+        <v>166</v>
+      </c>
       <c r="N18" s="82"/>
       <c r="O18" s="83"/>
       <c r="P18" s="83"/>
       <c r="Q18" s="84"/>
       <c r="R18" s="84">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="R18:R25" si="0">P18-Q18</f>
         <v>0</v>
       </c>
       <c r="S18" s="85"/>
@@ -3539,7 +3448,7 @@
       <c r="U18" s="83"/>
       <c r="V18" s="84"/>
       <c r="W18" s="86">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="W18:W25" si="1">U18-V18</f>
         <v>0</v>
       </c>
       <c r="X18" s="87"/>
@@ -3547,7 +3456,7 @@
       <c r="Z18" s="83"/>
       <c r="AA18" s="84"/>
       <c r="AB18" s="86">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="AB18:AB25" si="2">Z18-AA18</f>
         <v>0</v>
       </c>
       <c r="AC18" s="87"/>
@@ -3555,7 +3464,7 @@
       <c r="AE18" s="83"/>
       <c r="AF18" s="84"/>
       <c r="AG18" s="86">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="AG18:AG25" si="3">AE18-AF18</f>
         <v>0</v>
       </c>
       <c r="AH18" s="87"/>
@@ -3563,7 +3472,7 @@
       <c r="AJ18" s="83"/>
       <c r="AK18" s="84"/>
       <c r="AL18" s="86">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="AL18:AL25" si="4">AJ18-AK18</f>
         <v>0</v>
       </c>
       <c r="AM18" s="87"/>
@@ -3571,7 +3480,7 @@
       <c r="AO18" s="83"/>
       <c r="AP18" s="84"/>
       <c r="AQ18" s="86">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="AQ18:AQ25" si="5">AO18-AP18</f>
         <v>0</v>
       </c>
       <c r="AR18" s="87"/>
@@ -3579,7 +3488,7 @@
       <c r="AT18" s="83"/>
       <c r="AU18" s="84"/>
       <c r="AV18" s="86">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="AV18:AV25" si="6">AT18-AU18</f>
         <v>0</v>
       </c>
       <c r="AW18" s="87"/>
@@ -3587,7 +3496,7 @@
       <c r="AY18" s="83"/>
       <c r="AZ18" s="84"/>
       <c r="BA18" s="86">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="BA18:BA25" si="7">AY18-AZ18</f>
         <v>0</v>
       </c>
       <c r="BB18" s="87"/>
@@ -3595,7 +3504,7 @@
       <c r="BD18" s="83"/>
       <c r="BE18" s="84"/>
       <c r="BF18" s="86">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="BF18:BF25" si="8">BD18-BE18</f>
         <v>0</v>
       </c>
       <c r="BG18" s="87"/>
@@ -3603,7 +3512,7 @@
       <c r="BI18" s="83"/>
       <c r="BJ18" s="84"/>
       <c r="BK18" s="86">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="BK18:BK25" si="9">BI18-BJ18</f>
         <v>0</v>
       </c>
       <c r="BL18" s="87"/>
@@ -3611,7 +3520,7 @@
       <c r="BN18" s="83"/>
       <c r="BO18" s="84"/>
       <c r="BP18" s="86">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="BP18:BP25" si="10">BN18-BO18</f>
         <v>0</v>
       </c>
       <c r="BQ18" s="87"/>
@@ -3619,7 +3528,7 @@
       <c r="BS18" s="83"/>
       <c r="BT18" s="84"/>
       <c r="BU18" s="86">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="BU18:BU25" si="11">BS18-BT18</f>
         <v>0</v>
       </c>
       <c r="BV18" s="85">
@@ -3628,46 +3537,30 @@
       <c r="BW18" s="89"/>
       <c r="BX18" s="90"/>
     </row>
-    <row r="19" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:139" x14ac:dyDescent="0.25">
       <c r="A19" s="91" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B19" s="83">
-        <v>9501215650</v>
+        <v>9501079958</v>
       </c>
       <c r="C19" s="98">
-        <v>46065</v>
+        <v>45931</v>
       </c>
       <c r="D19" s="98">
-        <v>46387</v>
+        <v>46265</v>
       </c>
       <c r="E19" s="92" t="s">
-        <v>108</v>
-      </c>
-      <c r="F19" s="92" t="s">
-        <v>109</v>
-      </c>
-      <c r="G19" s="92">
-        <v>41500000</v>
-      </c>
-      <c r="H19" s="92">
-        <v>1400</v>
-      </c>
-      <c r="I19" s="92" t="s">
-        <v>105</v>
-      </c>
-      <c r="J19" s="92">
-        <v>2340693</v>
-      </c>
-      <c r="K19" s="99">
-        <v>54880</v>
-      </c>
-      <c r="L19" s="104" t="s">
-        <v>169</v>
-      </c>
-      <c r="M19" s="103" t="s">
-        <v>166</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="F19" s="92"/>
+      <c r="G19" s="92"/>
+      <c r="H19" s="92"/>
+      <c r="I19" s="92"/>
+      <c r="J19" s="92"/>
+      <c r="K19" s="93"/>
+      <c r="L19" s="104"/>
+      <c r="M19" s="103"/>
       <c r="N19" s="82"/>
       <c r="O19" s="83"/>
       <c r="P19" s="83"/>
@@ -3770,28 +3663,46 @@
       <c r="BW19" s="89"/>
       <c r="BX19" s="90"/>
     </row>
-    <row r="20" spans="1:76" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="91"/>
-      <c r="B20" s="83" t="s">
-        <v>110</v>
-      </c>
-      <c r="C20" s="92"/>
-      <c r="D20" s="92"/>
-      <c r="E20" s="92"/>
+    <row r="20" spans="1:139" x14ac:dyDescent="0.25">
+      <c r="A20" s="91" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" s="83">
+        <v>9501215650</v>
+      </c>
+      <c r="C20" s="98">
+        <v>46065</v>
+      </c>
+      <c r="D20" s="98">
+        <v>46387</v>
+      </c>
+      <c r="E20" s="92" t="s">
+        <v>108</v>
+      </c>
       <c r="F20" s="92" t="s">
-        <v>111</v>
-      </c>
-      <c r="G20" s="92"/>
-      <c r="H20" s="92"/>
-      <c r="I20" s="92"/>
-      <c r="J20" s="92"/>
+        <v>109</v>
+      </c>
+      <c r="G20" s="92">
+        <v>41500000</v>
+      </c>
+      <c r="H20" s="92">
+        <v>1400</v>
+      </c>
+      <c r="I20" s="92" t="s">
+        <v>105</v>
+      </c>
+      <c r="J20" s="92">
+        <v>2340693</v>
+      </c>
       <c r="K20" s="99">
-        <v>150000</v>
-      </c>
-      <c r="L20" s="102" t="s">
-        <v>170</v>
-      </c>
-      <c r="M20" s="103"/>
+        <v>54880</v>
+      </c>
+      <c r="L20" s="104" t="s">
+        <v>169</v>
+      </c>
+      <c r="M20" s="103" t="s">
+        <v>166</v>
+      </c>
       <c r="N20" s="82"/>
       <c r="O20" s="83"/>
       <c r="P20" s="83"/>
@@ -3894,34 +3805,26 @@
       <c r="BW20" s="89"/>
       <c r="BX20" s="90"/>
     </row>
-    <row r="21" spans="1:76" x14ac:dyDescent="0.25">
-      <c r="A21" s="91" t="s">
-        <v>112</v>
-      </c>
-      <c r="B21" s="83"/>
+    <row r="21" spans="1:139" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="91"/>
+      <c r="B21" s="83" t="s">
+        <v>110</v>
+      </c>
       <c r="C21" s="92"/>
       <c r="D21" s="92"/>
-      <c r="E21" s="92" t="s">
-        <v>101</v>
-      </c>
+      <c r="E21" s="92"/>
       <c r="F21" s="92" t="s">
-        <v>102</v>
-      </c>
-      <c r="G21" s="92">
-        <v>41500000</v>
-      </c>
-      <c r="H21" s="92">
-        <v>1400</v>
-      </c>
-      <c r="I21" s="92" t="s">
-        <v>105</v>
-      </c>
-      <c r="J21" s="92">
-        <v>2321403</v>
-      </c>
-      <c r="K21" s="93"/>
+        <v>111</v>
+      </c>
+      <c r="G21" s="92"/>
+      <c r="H21" s="92"/>
+      <c r="I21" s="92"/>
+      <c r="J21" s="92"/>
+      <c r="K21" s="99">
+        <v>150000</v>
+      </c>
       <c r="L21" s="102" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="M21" s="103"/>
       <c r="N21" s="82"/>
@@ -4026,22 +3929,34 @@
       <c r="BW21" s="89"/>
       <c r="BX21" s="90"/>
     </row>
-    <row r="22" spans="1:76" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="91"/>
+    <row r="22" spans="1:139" x14ac:dyDescent="0.25">
+      <c r="A22" s="91" t="s">
+        <v>112</v>
+      </c>
       <c r="B22" s="83"/>
       <c r="C22" s="92"/>
       <c r="D22" s="92"/>
-      <c r="E22" s="92"/>
+      <c r="E22" s="92" t="s">
+        <v>101</v>
+      </c>
       <c r="F22" s="92" t="s">
-        <v>113</v>
-      </c>
-      <c r="G22" s="92"/>
-      <c r="H22" s="92"/>
-      <c r="I22" s="92"/>
-      <c r="J22" s="92"/>
+        <v>102</v>
+      </c>
+      <c r="G22" s="92">
+        <v>41500000</v>
+      </c>
+      <c r="H22" s="92">
+        <v>1400</v>
+      </c>
+      <c r="I22" s="92" t="s">
+        <v>105</v>
+      </c>
+      <c r="J22" s="92">
+        <v>2321403</v>
+      </c>
       <c r="K22" s="93"/>
       <c r="L22" s="102" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="M22" s="103"/>
       <c r="N22" s="82"/>
@@ -4146,14 +4061,14 @@
       <c r="BW22" s="89"/>
       <c r="BX22" s="90"/>
     </row>
-    <row r="23" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:139" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="91"/>
       <c r="B23" s="83"/>
       <c r="C23" s="92"/>
       <c r="D23" s="92"/>
       <c r="E23" s="92"/>
       <c r="F23" s="92" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G23" s="92"/>
       <c r="H23" s="92"/>
@@ -4161,7 +4076,7 @@
       <c r="J23" s="92"/>
       <c r="K23" s="93"/>
       <c r="L23" s="102" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M23" s="103"/>
       <c r="N23" s="82"/>
@@ -4266,14 +4181,14 @@
       <c r="BW23" s="89"/>
       <c r="BX23" s="90"/>
     </row>
-    <row r="24" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:139" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="91"/>
       <c r="B24" s="83"/>
       <c r="C24" s="92"/>
       <c r="D24" s="92"/>
       <c r="E24" s="92"/>
       <c r="F24" s="92" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G24" s="92"/>
       <c r="H24" s="92"/>
@@ -4281,7 +4196,7 @@
       <c r="J24" s="92"/>
       <c r="K24" s="93"/>
       <c r="L24" s="102" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="M24" s="103"/>
       <c r="N24" s="82"/>
@@ -4386,14 +4301,14 @@
       <c r="BW24" s="89"/>
       <c r="BX24" s="90"/>
     </row>
-    <row r="25" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:139" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="91"/>
       <c r="B25" s="83"/>
       <c r="C25" s="92"/>
       <c r="D25" s="92"/>
       <c r="E25" s="92"/>
       <c r="F25" s="92" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G25" s="92"/>
       <c r="H25" s="92"/>
@@ -4401,7 +4316,7 @@
       <c r="J25" s="92"/>
       <c r="K25" s="93"/>
       <c r="L25" s="102" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M25" s="103"/>
       <c r="N25" s="82"/>
@@ -4409,7 +4324,7 @@
       <c r="P25" s="83"/>
       <c r="Q25" s="84"/>
       <c r="R25" s="84">
-        <f t="shared" ref="R25:R29" si="12">P25-Q25</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S25" s="85"/>
@@ -4417,7 +4332,7 @@
       <c r="U25" s="83"/>
       <c r="V25" s="84"/>
       <c r="W25" s="86">
-        <f t="shared" ref="W25:W29" si="13">U25-V25</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X25" s="87"/>
@@ -4425,7 +4340,7 @@
       <c r="Z25" s="83"/>
       <c r="AA25" s="84"/>
       <c r="AB25" s="86">
-        <f t="shared" ref="AB25:AB29" si="14">Z25-AA25</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AC25" s="87"/>
@@ -4433,7 +4348,7 @@
       <c r="AE25" s="83"/>
       <c r="AF25" s="84"/>
       <c r="AG25" s="86">
-        <f t="shared" ref="AG25:AG29" si="15">AE25-AF25</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AH25" s="87"/>
@@ -4441,7 +4356,7 @@
       <c r="AJ25" s="83"/>
       <c r="AK25" s="84"/>
       <c r="AL25" s="86">
-        <f t="shared" ref="AL25:AL29" si="16">AJ25-AK25</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AM25" s="87"/>
@@ -4449,7 +4364,7 @@
       <c r="AO25" s="83"/>
       <c r="AP25" s="84"/>
       <c r="AQ25" s="86">
-        <f t="shared" ref="AQ25:AQ29" si="17">AO25-AP25</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AR25" s="87"/>
@@ -4457,7 +4372,7 @@
       <c r="AT25" s="83"/>
       <c r="AU25" s="84"/>
       <c r="AV25" s="86">
-        <f t="shared" ref="AV25:AV29" si="18">AT25-AU25</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AW25" s="87"/>
@@ -4465,7 +4380,7 @@
       <c r="AY25" s="83"/>
       <c r="AZ25" s="84"/>
       <c r="BA25" s="86">
-        <f t="shared" ref="BA25:BA29" si="19">AY25-AZ25</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="BB25" s="87"/>
@@ -4473,7 +4388,7 @@
       <c r="BD25" s="83"/>
       <c r="BE25" s="84"/>
       <c r="BF25" s="86">
-        <f t="shared" ref="BF25:BF29" si="20">BD25-BE25</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="BG25" s="87"/>
@@ -4481,7 +4396,7 @@
       <c r="BI25" s="83"/>
       <c r="BJ25" s="84"/>
       <c r="BK25" s="86">
-        <f t="shared" ref="BK25:BK29" si="21">BI25-BJ25</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="BL25" s="87"/>
@@ -4489,7 +4404,7 @@
       <c r="BN25" s="83"/>
       <c r="BO25" s="84"/>
       <c r="BP25" s="86">
-        <f t="shared" ref="BP25:BP29" si="22">BN25-BO25</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BQ25" s="87"/>
@@ -4497,7 +4412,7 @@
       <c r="BS25" s="83"/>
       <c r="BT25" s="84"/>
       <c r="BU25" s="86">
-        <f t="shared" ref="BU25:BU29" si="23">BS25-BT25</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="BV25" s="85">
@@ -4506,14 +4421,14 @@
       <c r="BW25" s="89"/>
       <c r="BX25" s="90"/>
     </row>
-    <row r="26" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:139" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="91"/>
       <c r="B26" s="83"/>
       <c r="C26" s="92"/>
       <c r="D26" s="92"/>
       <c r="E26" s="92"/>
       <c r="F26" s="92" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G26" s="92"/>
       <c r="H26" s="92"/>
@@ -4521,7 +4436,7 @@
       <c r="J26" s="92"/>
       <c r="K26" s="93"/>
       <c r="L26" s="102" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="M26" s="103"/>
       <c r="N26" s="82"/>
@@ -4529,7 +4444,7 @@
       <c r="P26" s="83"/>
       <c r="Q26" s="84"/>
       <c r="R26" s="84">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="R26:R30" si="12">P26-Q26</f>
         <v>0</v>
       </c>
       <c r="S26" s="85"/>
@@ -4537,7 +4452,7 @@
       <c r="U26" s="83"/>
       <c r="V26" s="84"/>
       <c r="W26" s="86">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="W26:W30" si="13">U26-V26</f>
         <v>0</v>
       </c>
       <c r="X26" s="87"/>
@@ -4545,7 +4460,7 @@
       <c r="Z26" s="83"/>
       <c r="AA26" s="84"/>
       <c r="AB26" s="86">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="AB26:AB30" si="14">Z26-AA26</f>
         <v>0</v>
       </c>
       <c r="AC26" s="87"/>
@@ -4553,7 +4468,7 @@
       <c r="AE26" s="83"/>
       <c r="AF26" s="84"/>
       <c r="AG26" s="86">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="AG26:AG30" si="15">AE26-AF26</f>
         <v>0</v>
       </c>
       <c r="AH26" s="87"/>
@@ -4561,7 +4476,7 @@
       <c r="AJ26" s="83"/>
       <c r="AK26" s="84"/>
       <c r="AL26" s="86">
-        <f t="shared" si="16"/>
+        <f t="shared" ref="AL26:AL30" si="16">AJ26-AK26</f>
         <v>0</v>
       </c>
       <c r="AM26" s="87"/>
@@ -4569,7 +4484,7 @@
       <c r="AO26" s="83"/>
       <c r="AP26" s="84"/>
       <c r="AQ26" s="86">
-        <f t="shared" si="17"/>
+        <f t="shared" ref="AQ26:AQ30" si="17">AO26-AP26</f>
         <v>0</v>
       </c>
       <c r="AR26" s="87"/>
@@ -4577,7 +4492,7 @@
       <c r="AT26" s="83"/>
       <c r="AU26" s="84"/>
       <c r="AV26" s="86">
-        <f t="shared" si="18"/>
+        <f t="shared" ref="AV26:AV30" si="18">AT26-AU26</f>
         <v>0</v>
       </c>
       <c r="AW26" s="87"/>
@@ -4585,7 +4500,7 @@
       <c r="AY26" s="83"/>
       <c r="AZ26" s="84"/>
       <c r="BA26" s="86">
-        <f t="shared" si="19"/>
+        <f t="shared" ref="BA26:BA30" si="19">AY26-AZ26</f>
         <v>0</v>
       </c>
       <c r="BB26" s="87"/>
@@ -4593,7 +4508,7 @@
       <c r="BD26" s="83"/>
       <c r="BE26" s="84"/>
       <c r="BF26" s="86">
-        <f t="shared" si="20"/>
+        <f t="shared" ref="BF26:BF30" si="20">BD26-BE26</f>
         <v>0</v>
       </c>
       <c r="BG26" s="87"/>
@@ -4601,7 +4516,7 @@
       <c r="BI26" s="83"/>
       <c r="BJ26" s="84"/>
       <c r="BK26" s="86">
-        <f t="shared" si="21"/>
+        <f t="shared" ref="BK26:BK30" si="21">BI26-BJ26</f>
         <v>0</v>
       </c>
       <c r="BL26" s="87"/>
@@ -4609,7 +4524,7 @@
       <c r="BN26" s="83"/>
       <c r="BO26" s="84"/>
       <c r="BP26" s="86">
-        <f t="shared" si="22"/>
+        <f t="shared" ref="BP26:BP30" si="22">BN26-BO26</f>
         <v>0</v>
       </c>
       <c r="BQ26" s="87"/>
@@ -4617,7 +4532,7 @@
       <c r="BS26" s="83"/>
       <c r="BT26" s="84"/>
       <c r="BU26" s="86">
-        <f t="shared" si="23"/>
+        <f t="shared" ref="BU26:BU30" si="23">BS26-BT26</f>
         <v>0</v>
       </c>
       <c r="BV26" s="85">
@@ -4626,14 +4541,14 @@
       <c r="BW26" s="89"/>
       <c r="BX26" s="90"/>
     </row>
-    <row r="27" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:139" x14ac:dyDescent="0.25">
       <c r="A27" s="91"/>
       <c r="B27" s="83"/>
       <c r="C27" s="92"/>
       <c r="D27" s="92"/>
       <c r="E27" s="92"/>
       <c r="F27" s="92" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G27" s="92"/>
       <c r="H27" s="92"/>
@@ -4641,7 +4556,7 @@
       <c r="J27" s="92"/>
       <c r="K27" s="93"/>
       <c r="L27" s="102" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M27" s="103"/>
       <c r="N27" s="82"/>
@@ -4746,14 +4661,14 @@
       <c r="BW27" s="89"/>
       <c r="BX27" s="90"/>
     </row>
-    <row r="28" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:139" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="91"/>
       <c r="B28" s="83"/>
       <c r="C28" s="92"/>
       <c r="D28" s="92"/>
       <c r="E28" s="92"/>
       <c r="F28" s="92" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G28" s="92"/>
       <c r="H28" s="92"/>
@@ -4761,7 +4676,7 @@
       <c r="J28" s="92"/>
       <c r="K28" s="93"/>
       <c r="L28" s="102" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="M28" s="103"/>
       <c r="N28" s="82"/>
@@ -4866,14 +4781,14 @@
       <c r="BW28" s="89"/>
       <c r="BX28" s="90"/>
     </row>
-    <row r="29" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:139" x14ac:dyDescent="0.25">
       <c r="A29" s="91"/>
       <c r="B29" s="83"/>
       <c r="C29" s="92"/>
       <c r="D29" s="92"/>
       <c r="E29" s="92"/>
       <c r="F29" s="92" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G29" s="92"/>
       <c r="H29" s="92"/>
@@ -4986,14 +4901,14 @@
       <c r="BW29" s="89"/>
       <c r="BX29" s="90"/>
     </row>
-    <row r="30" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:139" x14ac:dyDescent="0.25">
       <c r="A30" s="91"/>
       <c r="B30" s="83"/>
       <c r="C30" s="92"/>
       <c r="D30" s="92"/>
       <c r="E30" s="92"/>
       <c r="F30" s="92" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G30" s="92"/>
       <c r="H30" s="92"/>
@@ -5001,7 +4916,7 @@
       <c r="J30" s="92"/>
       <c r="K30" s="93"/>
       <c r="L30" s="102" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="M30" s="103"/>
       <c r="N30" s="82"/>
@@ -5009,7 +4924,7 @@
       <c r="P30" s="83"/>
       <c r="Q30" s="84"/>
       <c r="R30" s="84">
-        <f t="shared" ref="R30:R64" si="24">P30-Q30</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="S30" s="85"/>
@@ -5017,7 +4932,7 @@
       <c r="U30" s="83"/>
       <c r="V30" s="84"/>
       <c r="W30" s="86">
-        <f t="shared" ref="W30:W64" si="25">U30-V30</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="X30" s="87"/>
@@ -5025,7 +4940,7 @@
       <c r="Z30" s="83"/>
       <c r="AA30" s="84"/>
       <c r="AB30" s="86">
-        <f t="shared" ref="AB30:AB64" si="26">Z30-AA30</f>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AC30" s="87"/>
@@ -5033,7 +4948,7 @@
       <c r="AE30" s="83"/>
       <c r="AF30" s="84"/>
       <c r="AG30" s="86">
-        <f t="shared" ref="AG30:AG64" si="27">AE30-AF30</f>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AH30" s="87"/>
@@ -5041,7 +4956,7 @@
       <c r="AJ30" s="83"/>
       <c r="AK30" s="84"/>
       <c r="AL30" s="86">
-        <f t="shared" ref="AL30:AL64" si="28">AJ30-AK30</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AM30" s="87"/>
@@ -5049,7 +4964,7 @@
       <c r="AO30" s="83"/>
       <c r="AP30" s="84"/>
       <c r="AQ30" s="86">
-        <f t="shared" ref="AQ30:AQ64" si="29">AO30-AP30</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AR30" s="87"/>
@@ -5057,7 +4972,7 @@
       <c r="AT30" s="83"/>
       <c r="AU30" s="84"/>
       <c r="AV30" s="86">
-        <f t="shared" ref="AV30:AV64" si="30">AT30-AU30</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="AW30" s="87"/>
@@ -5065,7 +4980,7 @@
       <c r="AY30" s="83"/>
       <c r="AZ30" s="84"/>
       <c r="BA30" s="86">
-        <f t="shared" ref="BA30:BA64" si="31">AY30-AZ30</f>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="BB30" s="87"/>
@@ -5073,7 +4988,7 @@
       <c r="BD30" s="83"/>
       <c r="BE30" s="84"/>
       <c r="BF30" s="86">
-        <f t="shared" ref="BF30:BF64" si="32">BD30-BE30</f>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="BG30" s="87"/>
@@ -5081,7 +4996,7 @@
       <c r="BI30" s="83"/>
       <c r="BJ30" s="84"/>
       <c r="BK30" s="86">
-        <f t="shared" ref="BK30:BK64" si="33">BI30-BJ30</f>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="BL30" s="87"/>
@@ -5089,7 +5004,7 @@
       <c r="BN30" s="83"/>
       <c r="BO30" s="84"/>
       <c r="BP30" s="86">
-        <f t="shared" ref="BP30:BP64" si="34">BN30-BO30</f>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="BQ30" s="87"/>
@@ -5097,7 +5012,7 @@
       <c r="BS30" s="83"/>
       <c r="BT30" s="84"/>
       <c r="BU30" s="86">
-        <f t="shared" ref="BU30:BU64" si="35">BS30-BT30</f>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BV30" s="85">
@@ -5106,14 +5021,14 @@
       <c r="BW30" s="89"/>
       <c r="BX30" s="90"/>
     </row>
-    <row r="31" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:139" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="91"/>
       <c r="B31" s="83"/>
       <c r="C31" s="92"/>
       <c r="D31" s="92"/>
       <c r="E31" s="92"/>
       <c r="F31" s="92" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G31" s="92"/>
       <c r="H31" s="92"/>
@@ -5121,7 +5036,7 @@
       <c r="J31" s="92"/>
       <c r="K31" s="93"/>
       <c r="L31" s="102" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="M31" s="103"/>
       <c r="N31" s="82"/>
@@ -5129,7 +5044,7 @@
       <c r="P31" s="83"/>
       <c r="Q31" s="84"/>
       <c r="R31" s="84">
-        <f t="shared" si="24"/>
+        <f t="shared" ref="R31:R65" si="24">P31-Q31</f>
         <v>0</v>
       </c>
       <c r="S31" s="85"/>
@@ -5137,7 +5052,7 @@
       <c r="U31" s="83"/>
       <c r="V31" s="84"/>
       <c r="W31" s="86">
-        <f t="shared" si="25"/>
+        <f t="shared" ref="W31:W65" si="25">U31-V31</f>
         <v>0</v>
       </c>
       <c r="X31" s="87"/>
@@ -5145,7 +5060,7 @@
       <c r="Z31" s="83"/>
       <c r="AA31" s="84"/>
       <c r="AB31" s="86">
-        <f t="shared" si="26"/>
+        <f t="shared" ref="AB31:AB65" si="26">Z31-AA31</f>
         <v>0</v>
       </c>
       <c r="AC31" s="87"/>
@@ -5153,7 +5068,7 @@
       <c r="AE31" s="83"/>
       <c r="AF31" s="84"/>
       <c r="AG31" s="86">
-        <f t="shared" si="27"/>
+        <f t="shared" ref="AG31:AG65" si="27">AE31-AF31</f>
         <v>0</v>
       </c>
       <c r="AH31" s="87"/>
@@ -5161,7 +5076,7 @@
       <c r="AJ31" s="83"/>
       <c r="AK31" s="84"/>
       <c r="AL31" s="86">
-        <f t="shared" si="28"/>
+        <f t="shared" ref="AL31:AL65" si="28">AJ31-AK31</f>
         <v>0</v>
       </c>
       <c r="AM31" s="87"/>
@@ -5169,7 +5084,7 @@
       <c r="AO31" s="83"/>
       <c r="AP31" s="84"/>
       <c r="AQ31" s="86">
-        <f t="shared" si="29"/>
+        <f t="shared" ref="AQ31:AQ65" si="29">AO31-AP31</f>
         <v>0</v>
       </c>
       <c r="AR31" s="87"/>
@@ -5177,7 +5092,7 @@
       <c r="AT31" s="83"/>
       <c r="AU31" s="84"/>
       <c r="AV31" s="86">
-        <f t="shared" si="30"/>
+        <f t="shared" ref="AV31:AV65" si="30">AT31-AU31</f>
         <v>0</v>
       </c>
       <c r="AW31" s="87"/>
@@ -5185,7 +5100,7 @@
       <c r="AY31" s="83"/>
       <c r="AZ31" s="84"/>
       <c r="BA31" s="86">
-        <f t="shared" si="31"/>
+        <f t="shared" ref="BA31:BA65" si="31">AY31-AZ31</f>
         <v>0</v>
       </c>
       <c r="BB31" s="87"/>
@@ -5193,7 +5108,7 @@
       <c r="BD31" s="83"/>
       <c r="BE31" s="84"/>
       <c r="BF31" s="86">
-        <f t="shared" si="32"/>
+        <f t="shared" ref="BF31:BF65" si="32">BD31-BE31</f>
         <v>0</v>
       </c>
       <c r="BG31" s="87"/>
@@ -5201,7 +5116,7 @@
       <c r="BI31" s="83"/>
       <c r="BJ31" s="84"/>
       <c r="BK31" s="86">
-        <f t="shared" si="33"/>
+        <f t="shared" ref="BK31:BK65" si="33">BI31-BJ31</f>
         <v>0</v>
       </c>
       <c r="BL31" s="87"/>
@@ -5209,7 +5124,7 @@
       <c r="BN31" s="83"/>
       <c r="BO31" s="84"/>
       <c r="BP31" s="86">
-        <f t="shared" si="34"/>
+        <f t="shared" ref="BP31:BP65" si="34">BN31-BO31</f>
         <v>0</v>
       </c>
       <c r="BQ31" s="87"/>
@@ -5217,7 +5132,7 @@
       <c r="BS31" s="83"/>
       <c r="BT31" s="84"/>
       <c r="BU31" s="86">
-        <f t="shared" si="35"/>
+        <f t="shared" ref="BU31:BU65" si="35">BS31-BT31</f>
         <v>0</v>
       </c>
       <c r="BV31" s="85">
@@ -5226,14 +5141,14 @@
       <c r="BW31" s="89"/>
       <c r="BX31" s="90"/>
     </row>
-    <row r="32" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:139" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="91"/>
       <c r="B32" s="83"/>
       <c r="C32" s="92"/>
       <c r="D32" s="92"/>
       <c r="E32" s="92"/>
       <c r="F32" s="92" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G32" s="92"/>
       <c r="H32" s="92"/>
@@ -5241,7 +5156,7 @@
       <c r="J32" s="92"/>
       <c r="K32" s="93"/>
       <c r="L32" s="102" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="M32" s="103"/>
       <c r="N32" s="82"/>
@@ -5346,14 +5261,14 @@
       <c r="BW32" s="89"/>
       <c r="BX32" s="90"/>
     </row>
-    <row r="33" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:76" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="91"/>
       <c r="B33" s="83"/>
       <c r="C33" s="92"/>
       <c r="D33" s="92"/>
       <c r="E33" s="92"/>
       <c r="F33" s="92" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G33" s="92"/>
       <c r="H33" s="92"/>
@@ -5361,7 +5276,7 @@
       <c r="J33" s="92"/>
       <c r="K33" s="93"/>
       <c r="L33" s="102" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M33" s="103"/>
       <c r="N33" s="82"/>
@@ -5466,14 +5381,14 @@
       <c r="BW33" s="89"/>
       <c r="BX33" s="90"/>
     </row>
-    <row r="34" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A34" s="91"/>
       <c r="B34" s="83"/>
       <c r="C34" s="92"/>
       <c r="D34" s="92"/>
       <c r="E34" s="92"/>
       <c r="F34" s="92" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G34" s="92"/>
       <c r="H34" s="92"/>
@@ -5481,7 +5396,7 @@
       <c r="J34" s="92"/>
       <c r="K34" s="93"/>
       <c r="L34" s="102" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="M34" s="103"/>
       <c r="N34" s="82"/>
@@ -5586,14 +5501,14 @@
       <c r="BW34" s="89"/>
       <c r="BX34" s="90"/>
     </row>
-    <row r="35" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="91"/>
       <c r="B35" s="83"/>
       <c r="C35" s="92"/>
       <c r="D35" s="92"/>
       <c r="E35" s="92"/>
       <c r="F35" s="92" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G35" s="92"/>
       <c r="H35" s="92"/>
@@ -5601,7 +5516,7 @@
       <c r="J35" s="92"/>
       <c r="K35" s="93"/>
       <c r="L35" s="102" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="M35" s="103"/>
       <c r="N35" s="82"/>
@@ -5713,7 +5628,7 @@
       <c r="D36" s="92"/>
       <c r="E36" s="92"/>
       <c r="F36" s="92" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G36" s="92"/>
       <c r="H36" s="92"/>
@@ -5721,7 +5636,7 @@
       <c r="J36" s="92"/>
       <c r="K36" s="93"/>
       <c r="L36" s="102" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="M36" s="103"/>
       <c r="N36" s="82"/>
@@ -5833,7 +5748,7 @@
       <c r="D37" s="92"/>
       <c r="E37" s="92"/>
       <c r="F37" s="92" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G37" s="92"/>
       <c r="H37" s="92"/>
@@ -5841,7 +5756,7 @@
       <c r="J37" s="92"/>
       <c r="K37" s="93"/>
       <c r="L37" s="102" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M37" s="103"/>
       <c r="N37" s="82"/>
@@ -5953,7 +5868,7 @@
       <c r="D38" s="92"/>
       <c r="E38" s="92"/>
       <c r="F38" s="92" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="G38" s="92"/>
       <c r="H38" s="92"/>
@@ -5961,7 +5876,7 @@
       <c r="J38" s="92"/>
       <c r="K38" s="93"/>
       <c r="L38" s="102" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M38" s="103"/>
       <c r="N38" s="82"/>
@@ -6066,14 +5981,14 @@
       <c r="BW38" s="89"/>
       <c r="BX38" s="90"/>
     </row>
-    <row r="39" spans="1:76" ht="60" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A39" s="91"/>
       <c r="B39" s="83"/>
       <c r="C39" s="92"/>
       <c r="D39" s="92"/>
       <c r="E39" s="92"/>
       <c r="F39" s="92" t="s">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="G39" s="92"/>
       <c r="H39" s="92"/>
@@ -6081,7 +5996,7 @@
       <c r="J39" s="92"/>
       <c r="K39" s="93"/>
       <c r="L39" s="102" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M39" s="103"/>
       <c r="N39" s="82"/>
@@ -6186,14 +6101,14 @@
       <c r="BW39" s="89"/>
       <c r="BX39" s="90"/>
     </row>
-    <row r="40" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:76" ht="60" x14ac:dyDescent="0.25">
       <c r="A40" s="91"/>
       <c r="B40" s="83"/>
       <c r="C40" s="92"/>
       <c r="D40" s="92"/>
       <c r="E40" s="92"/>
       <c r="F40" s="92" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G40" s="92"/>
       <c r="H40" s="92"/>
@@ -6201,7 +6116,7 @@
       <c r="J40" s="92"/>
       <c r="K40" s="93"/>
       <c r="L40" s="102" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="M40" s="103"/>
       <c r="N40" s="82"/>
@@ -6306,14 +6221,14 @@
       <c r="BW40" s="89"/>
       <c r="BX40" s="90"/>
     </row>
-    <row r="41" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="91"/>
       <c r="B41" s="83"/>
       <c r="C41" s="92"/>
       <c r="D41" s="92"/>
       <c r="E41" s="92"/>
       <c r="F41" s="92" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G41" s="92"/>
       <c r="H41" s="92"/>
@@ -6321,7 +6236,7 @@
       <c r="J41" s="92"/>
       <c r="K41" s="93"/>
       <c r="L41" s="102" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="M41" s="103"/>
       <c r="N41" s="82"/>
@@ -6426,16 +6341,14 @@
       <c r="BW41" s="89"/>
       <c r="BX41" s="90"/>
     </row>
-    <row r="42" spans="1:76" ht="30" x14ac:dyDescent="0.25">
-      <c r="A42" s="91" t="s">
-        <v>132</v>
-      </c>
+    <row r="42" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+      <c r="A42" s="91"/>
       <c r="B42" s="83"/>
       <c r="C42" s="92"/>
       <c r="D42" s="92"/>
       <c r="E42" s="92"/>
       <c r="F42" s="92" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G42" s="92"/>
       <c r="H42" s="92"/>
@@ -6443,7 +6356,7 @@
       <c r="J42" s="92"/>
       <c r="K42" s="93"/>
       <c r="L42" s="102" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="M42" s="103"/>
       <c r="N42" s="82"/>
@@ -6550,14 +6463,14 @@
     </row>
     <row r="43" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="91" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B43" s="83"/>
       <c r="C43" s="92"/>
       <c r="D43" s="92"/>
       <c r="E43" s="92"/>
       <c r="F43" s="92" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G43" s="92"/>
       <c r="H43" s="92"/>
@@ -6565,7 +6478,7 @@
       <c r="J43" s="92"/>
       <c r="K43" s="93"/>
       <c r="L43" s="102" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="M43" s="103"/>
       <c r="N43" s="82"/>
@@ -6670,14 +6583,16 @@
       <c r="BW43" s="89"/>
       <c r="BX43" s="90"/>
     </row>
-    <row r="44" spans="1:76" x14ac:dyDescent="0.25">
-      <c r="A44" s="91"/>
+    <row r="44" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="91" t="s">
+        <v>134</v>
+      </c>
       <c r="B44" s="83"/>
       <c r="C44" s="92"/>
       <c r="D44" s="92"/>
       <c r="E44" s="92"/>
       <c r="F44" s="92" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G44" s="92"/>
       <c r="H44" s="92"/>
@@ -6685,7 +6600,7 @@
       <c r="J44" s="92"/>
       <c r="K44" s="93"/>
       <c r="L44" s="102" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M44" s="103"/>
       <c r="N44" s="82"/>
@@ -6797,7 +6712,7 @@
       <c r="D45" s="92"/>
       <c r="E45" s="92"/>
       <c r="F45" s="92" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G45" s="92"/>
       <c r="H45" s="92"/>
@@ -6805,7 +6720,7 @@
       <c r="J45" s="92"/>
       <c r="K45" s="93"/>
       <c r="L45" s="102" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="M45" s="103"/>
       <c r="N45" s="82"/>
@@ -6910,46 +6825,24 @@
       <c r="BW45" s="89"/>
       <c r="BX45" s="90"/>
     </row>
-    <row r="46" spans="1:76" ht="30" x14ac:dyDescent="0.25">
-      <c r="A46" s="91" t="s">
-        <v>138</v>
-      </c>
-      <c r="B46" s="83">
-        <v>9501137831</v>
-      </c>
-      <c r="C46" s="98">
-        <v>45992</v>
-      </c>
-      <c r="D46" s="98">
-        <v>46356</v>
-      </c>
-      <c r="E46" s="92" t="s">
-        <v>139</v>
-      </c>
+    <row r="46" spans="1:76" x14ac:dyDescent="0.25">
+      <c r="A46" s="91"/>
+      <c r="B46" s="83"/>
+      <c r="C46" s="92"/>
+      <c r="D46" s="92"/>
+      <c r="E46" s="92"/>
       <c r="F46" s="92" t="s">
-        <v>140</v>
-      </c>
-      <c r="G46" s="92">
-        <v>41010100</v>
-      </c>
-      <c r="H46" s="92">
-        <v>7280</v>
-      </c>
-      <c r="I46" s="92" t="s">
-        <v>141</v>
-      </c>
-      <c r="J46" s="92">
-        <v>2662855</v>
-      </c>
-      <c r="K46" s="99">
-        <v>38005</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="G46" s="92"/>
+      <c r="H46" s="92"/>
+      <c r="I46" s="92"/>
+      <c r="J46" s="92"/>
+      <c r="K46" s="93"/>
       <c r="L46" s="102" t="s">
-        <v>195</v>
-      </c>
-      <c r="M46" s="103" t="s">
-        <v>166</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="M46" s="103"/>
       <c r="N46" s="82"/>
       <c r="O46" s="83"/>
       <c r="P46" s="83"/>
@@ -7052,12 +6945,12 @@
       <c r="BW46" s="89"/>
       <c r="BX46" s="90"/>
     </row>
-    <row r="47" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="91" t="s">
-        <v>97</v>
+        <v>138</v>
       </c>
       <c r="B47" s="83">
-        <v>9501137269</v>
+        <v>9501137831</v>
       </c>
       <c r="C47" s="98">
         <v>45992</v>
@@ -7066,10 +6959,10 @@
         <v>46356</v>
       </c>
       <c r="E47" s="92" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F47" s="92" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G47" s="92">
         <v>41010100</v>
@@ -7084,10 +6977,10 @@
         <v>2662855</v>
       </c>
       <c r="K47" s="99">
-        <v>9980</v>
+        <v>38005</v>
       </c>
       <c r="L47" s="102" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M47" s="103" t="s">
         <v>166</v>
@@ -7194,26 +7087,46 @@
       <c r="BW47" s="89"/>
       <c r="BX47" s="90"/>
     </row>
-    <row r="48" spans="1:76" ht="30" x14ac:dyDescent="0.25">
-      <c r="A48" s="91"/>
-      <c r="B48" s="83"/>
-      <c r="C48" s="92"/>
-      <c r="D48" s="92"/>
-      <c r="E48" s="92"/>
+    <row r="48" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+      <c r="A48" s="91" t="s">
+        <v>97</v>
+      </c>
+      <c r="B48" s="83">
+        <v>9501137269</v>
+      </c>
+      <c r="C48" s="98">
+        <v>45992</v>
+      </c>
+      <c r="D48" s="98">
+        <v>46356</v>
+      </c>
+      <c r="E48" s="92" t="s">
+        <v>142</v>
+      </c>
       <c r="F48" s="92" t="s">
-        <v>144</v>
-      </c>
-      <c r="G48" s="92"/>
-      <c r="H48" s="92"/>
-      <c r="I48" s="92"/>
-      <c r="J48" s="92"/>
+        <v>143</v>
+      </c>
+      <c r="G48" s="92">
+        <v>41010100</v>
+      </c>
+      <c r="H48" s="92">
+        <v>7280</v>
+      </c>
+      <c r="I48" s="92" t="s">
+        <v>141</v>
+      </c>
+      <c r="J48" s="92">
+        <v>2662855</v>
+      </c>
       <c r="K48" s="99">
-        <v>12000</v>
+        <v>9980</v>
       </c>
       <c r="L48" s="102" t="s">
-        <v>197</v>
-      </c>
-      <c r="M48" s="103"/>
+        <v>196</v>
+      </c>
+      <c r="M48" s="103" t="s">
+        <v>166</v>
+      </c>
       <c r="N48" s="82"/>
       <c r="O48" s="83"/>
       <c r="P48" s="83"/>
@@ -7316,24 +7229,24 @@
       <c r="BW48" s="89"/>
       <c r="BX48" s="90"/>
     </row>
-    <row r="49" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="91"/>
       <c r="B49" s="83"/>
       <c r="C49" s="92"/>
       <c r="D49" s="92"/>
       <c r="E49" s="92"/>
       <c r="F49" s="92" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G49" s="92"/>
       <c r="H49" s="92"/>
       <c r="I49" s="92"/>
       <c r="J49" s="92"/>
       <c r="K49" s="99">
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="L49" s="102" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="M49" s="103"/>
       <c r="N49" s="82"/>
@@ -7438,46 +7351,26 @@
       <c r="BW49" s="89"/>
       <c r="BX49" s="90"/>
     </row>
-    <row r="50" spans="1:76" ht="30" x14ac:dyDescent="0.25">
-      <c r="A50" s="91" t="s">
-        <v>97</v>
-      </c>
-      <c r="B50" s="83">
-        <v>9501166164</v>
-      </c>
-      <c r="C50" s="98">
-        <v>46023</v>
-      </c>
-      <c r="D50" s="98">
-        <v>46387</v>
-      </c>
-      <c r="E50" s="92" t="s">
-        <v>146</v>
-      </c>
+    <row r="50" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+      <c r="A50" s="91"/>
+      <c r="B50" s="83"/>
+      <c r="C50" s="92"/>
+      <c r="D50" s="92"/>
+      <c r="E50" s="92"/>
       <c r="F50" s="92" t="s">
-        <v>147</v>
-      </c>
-      <c r="G50" s="92">
-        <v>41500000</v>
-      </c>
-      <c r="H50" s="92">
-        <v>1400</v>
-      </c>
-      <c r="I50" s="92" t="s">
-        <v>105</v>
-      </c>
-      <c r="J50" s="92">
-        <v>2321403</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="G50" s="92"/>
+      <c r="H50" s="92"/>
+      <c r="I50" s="92"/>
+      <c r="J50" s="92"/>
       <c r="K50" s="99">
-        <v>4651600</v>
+        <v>0</v>
       </c>
       <c r="L50" s="102" t="s">
-        <v>199</v>
-      </c>
-      <c r="M50" s="103" t="s">
-        <v>166</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="M50" s="103"/>
       <c r="N50" s="82"/>
       <c r="O50" s="83"/>
       <c r="P50" s="83"/>
@@ -7580,18 +7473,18 @@
       <c r="BW50" s="89"/>
       <c r="BX50" s="90"/>
     </row>
-    <row r="51" spans="1:76" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="91" t="s">
         <v>97</v>
       </c>
       <c r="B51" s="83">
-        <v>9501190667</v>
+        <v>9501166164</v>
       </c>
       <c r="C51" s="98">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="D51" s="98">
-        <v>46296</v>
+        <v>46387</v>
       </c>
       <c r="E51" s="92" t="s">
         <v>146</v>
@@ -7612,10 +7505,10 @@
         <v>2321403</v>
       </c>
       <c r="K51" s="99">
-        <v>62500</v>
+        <v>4651600</v>
       </c>
       <c r="L51" s="102" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="M51" s="103" t="s">
         <v>166</v>
@@ -7724,22 +7617,22 @@
     </row>
     <row r="52" spans="1:76" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="91" t="s">
-        <v>148</v>
+        <v>97</v>
       </c>
       <c r="B52" s="83">
-        <v>9501199822</v>
+        <v>9501190667</v>
       </c>
       <c r="C52" s="98">
-        <v>46023</v>
+        <v>45992</v>
       </c>
       <c r="D52" s="98">
-        <v>46387</v>
+        <v>46296</v>
       </c>
       <c r="E52" s="92" t="s">
         <v>146</v>
       </c>
       <c r="F52" s="92" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G52" s="92">
         <v>41500000</v>
@@ -7754,10 +7647,10 @@
         <v>2321403</v>
       </c>
       <c r="K52" s="99">
-        <v>1058400</v>
+        <v>62500</v>
       </c>
       <c r="L52" s="102" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="M52" s="103" t="s">
         <v>166</v>
@@ -7866,10 +7759,10 @@
     </row>
     <row r="53" spans="1:76" ht="45" x14ac:dyDescent="0.25">
       <c r="A53" s="91" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B53" s="83">
-        <v>9501199827</v>
+        <v>9501199822</v>
       </c>
       <c r="C53" s="98">
         <v>46023</v>
@@ -7896,10 +7789,10 @@
         <v>2321403</v>
       </c>
       <c r="K53" s="99">
-        <v>577400</v>
+        <v>1058400</v>
       </c>
       <c r="L53" s="102" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M53" s="103" t="s">
         <v>166</v>
@@ -8006,12 +7899,12 @@
       <c r="BW53" s="89"/>
       <c r="BX53" s="90"/>
     </row>
-    <row r="54" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:76" ht="45" x14ac:dyDescent="0.25">
       <c r="A54" s="91" t="s">
-        <v>97</v>
+        <v>150</v>
       </c>
       <c r="B54" s="83">
-        <v>9501195328</v>
+        <v>9501199827</v>
       </c>
       <c r="C54" s="98">
         <v>46023</v>
@@ -8023,7 +7916,7 @@
         <v>146</v>
       </c>
       <c r="F54" s="92" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="G54" s="92">
         <v>41500000</v>
@@ -8038,10 +7931,10 @@
         <v>2321403</v>
       </c>
       <c r="K54" s="99">
-        <v>36000</v>
+        <v>577400</v>
       </c>
       <c r="L54" s="102" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M54" s="103" t="s">
         <v>166</v>
@@ -8149,23 +8042,45 @@
       <c r="BX54" s="90"/>
     </row>
     <row r="55" spans="1:76" x14ac:dyDescent="0.25">
-      <c r="A55" s="91"/>
-      <c r="B55" s="83"/>
-      <c r="C55" s="92"/>
-      <c r="D55" s="92"/>
-      <c r="E55" s="92"/>
+      <c r="A55" s="91" t="s">
+        <v>97</v>
+      </c>
+      <c r="B55" s="83">
+        <v>9501195328</v>
+      </c>
+      <c r="C55" s="98">
+        <v>46023</v>
+      </c>
+      <c r="D55" s="98">
+        <v>46387</v>
+      </c>
+      <c r="E55" s="92" t="s">
+        <v>146</v>
+      </c>
       <c r="F55" s="92" t="s">
-        <v>152</v>
-      </c>
-      <c r="G55" s="92"/>
-      <c r="H55" s="92"/>
-      <c r="I55" s="92"/>
-      <c r="J55" s="92"/>
-      <c r="K55" s="93"/>
+        <v>151</v>
+      </c>
+      <c r="G55" s="92">
+        <v>41500000</v>
+      </c>
+      <c r="H55" s="92">
+        <v>1400</v>
+      </c>
+      <c r="I55" s="92" t="s">
+        <v>105</v>
+      </c>
+      <c r="J55" s="92">
+        <v>2321403</v>
+      </c>
+      <c r="K55" s="99">
+        <v>36000</v>
+      </c>
       <c r="L55" s="102" t="s">
-        <v>204</v>
-      </c>
-      <c r="M55" s="103"/>
+        <v>203</v>
+      </c>
+      <c r="M55" s="103" t="s">
+        <v>166</v>
+      </c>
       <c r="N55" s="82"/>
       <c r="O55" s="83"/>
       <c r="P55" s="83"/>
@@ -8275,7 +8190,7 @@
       <c r="D56" s="92"/>
       <c r="E56" s="92"/>
       <c r="F56" s="92" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G56" s="92"/>
       <c r="H56" s="92"/>
@@ -8283,7 +8198,7 @@
       <c r="J56" s="92"/>
       <c r="K56" s="93"/>
       <c r="L56" s="102" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M56" s="103"/>
       <c r="N56" s="82"/>
@@ -8389,45 +8304,23 @@
       <c r="BX56" s="90"/>
     </row>
     <row r="57" spans="1:76" x14ac:dyDescent="0.25">
-      <c r="A57" s="91" t="s">
-        <v>10</v>
-      </c>
-      <c r="B57" s="83">
-        <v>9501212179</v>
-      </c>
-      <c r="C57" s="98">
-        <v>46023</v>
-      </c>
-      <c r="D57" s="92" t="s">
-        <v>154</v>
-      </c>
-      <c r="E57" s="92" t="s">
-        <v>146</v>
-      </c>
+      <c r="A57" s="91"/>
+      <c r="B57" s="83"/>
+      <c r="C57" s="92"/>
+      <c r="D57" s="92"/>
+      <c r="E57" s="92"/>
       <c r="F57" s="92" t="s">
-        <v>155</v>
-      </c>
-      <c r="G57" s="92">
-        <v>41500000</v>
-      </c>
-      <c r="H57" s="92">
-        <v>1400</v>
-      </c>
-      <c r="I57" s="92" t="s">
-        <v>105</v>
-      </c>
-      <c r="J57" s="92">
-        <v>2321403</v>
-      </c>
-      <c r="K57" s="99">
-        <v>334732.5</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="G57" s="92"/>
+      <c r="H57" s="92"/>
+      <c r="I57" s="92"/>
+      <c r="J57" s="92"/>
+      <c r="K57" s="93"/>
       <c r="L57" s="102" t="s">
-        <v>206</v>
-      </c>
-      <c r="M57" s="103" t="s">
-        <v>166</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="M57" s="103"/>
       <c r="N57" s="82"/>
       <c r="O57" s="83"/>
       <c r="P57" s="83"/>
@@ -8530,24 +8423,24 @@
       <c r="BW57" s="89"/>
       <c r="BX57" s="90"/>
     </row>
-    <row r="58" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A58" s="91" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="B58" s="83">
-        <v>9501196824</v>
+        <v>9501212179</v>
       </c>
       <c r="C58" s="98">
         <v>46023</v>
       </c>
-      <c r="D58" s="98">
-        <v>46387</v>
+      <c r="D58" s="92" t="s">
+        <v>154</v>
       </c>
       <c r="E58" s="92" t="s">
         <v>146</v>
       </c>
       <c r="F58" s="92" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G58" s="92">
         <v>41500000</v>
@@ -8562,10 +8455,10 @@
         <v>2321403</v>
       </c>
       <c r="K58" s="99">
-        <v>433000</v>
+        <v>334732.5</v>
       </c>
       <c r="L58" s="102" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="M58" s="103" t="s">
         <v>166</v>
@@ -8674,10 +8567,10 @@
     </row>
     <row r="59" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="91" t="s">
-        <v>157</v>
+        <v>97</v>
       </c>
       <c r="B59" s="83">
-        <v>9501196865</v>
+        <v>9501196824</v>
       </c>
       <c r="C59" s="98">
         <v>46023</v>
@@ -8689,7 +8582,7 @@
         <v>146</v>
       </c>
       <c r="F59" s="92" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G59" s="92">
         <v>41500000</v>
@@ -8704,10 +8597,10 @@
         <v>2321403</v>
       </c>
       <c r="K59" s="99">
-        <v>335904</v>
+        <v>433000</v>
       </c>
       <c r="L59" s="102" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="M59" s="103" t="s">
         <v>166</v>
@@ -8816,10 +8709,10 @@
     </row>
     <row r="60" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="91" t="s">
-        <v>97</v>
+        <v>157</v>
       </c>
       <c r="B60" s="83">
-        <v>9501158806</v>
+        <v>9501196865</v>
       </c>
       <c r="C60" s="98">
         <v>46023</v>
@@ -8831,7 +8724,7 @@
         <v>146</v>
       </c>
       <c r="F60" s="92" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G60" s="92">
         <v>41500000</v>
@@ -8846,10 +8739,10 @@
         <v>2321403</v>
       </c>
       <c r="K60" s="99">
-        <v>376200</v>
+        <v>335904</v>
       </c>
       <c r="L60" s="102" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="M60" s="103" t="s">
         <v>166</v>
@@ -8958,10 +8851,10 @@
     </row>
     <row r="61" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="91" t="s">
-        <v>160</v>
+        <v>97</v>
       </c>
       <c r="B61" s="83">
-        <v>9501159633</v>
+        <v>9501158806</v>
       </c>
       <c r="C61" s="98">
         <v>46023</v>
@@ -8970,13 +8863,13 @@
         <v>46387</v>
       </c>
       <c r="E61" s="92" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="F61" s="92" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="G61" s="92">
-        <v>61010000</v>
+        <v>41500000</v>
       </c>
       <c r="H61" s="92">
         <v>1400</v>
@@ -8988,10 +8881,10 @@
         <v>2321403</v>
       </c>
       <c r="K61" s="99">
-        <v>146493</v>
+        <v>376200</v>
       </c>
       <c r="L61" s="102" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M61" s="103" t="s">
         <v>166</v>
@@ -9100,40 +8993,40 @@
     </row>
     <row r="62" spans="1:76" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="91" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B62" s="83">
-        <v>9501199250</v>
+        <v>9501159633</v>
       </c>
       <c r="C62" s="98">
-        <v>46054</v>
+        <v>46023</v>
       </c>
       <c r="D62" s="98">
-        <v>46418</v>
+        <v>46387</v>
       </c>
       <c r="E62" s="92" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="F62" s="92" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G62" s="92">
-        <v>41010100</v>
+        <v>61010000</v>
       </c>
       <c r="H62" s="92">
-        <v>7280</v>
+        <v>1400</v>
       </c>
       <c r="I62" s="92" t="s">
-        <v>141</v>
+        <v>105</v>
       </c>
       <c r="J62" s="92">
-        <v>2662855</v>
+        <v>2321403</v>
       </c>
       <c r="K62" s="99">
-        <v>69429</v>
+        <v>146493</v>
       </c>
       <c r="L62" s="102" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="M62" s="103" t="s">
         <v>166</v>
@@ -9240,20 +9133,46 @@
       <c r="BW62" s="89"/>
       <c r="BX62" s="90"/>
     </row>
-    <row r="63" spans="1:76" x14ac:dyDescent="0.25">
-      <c r="A63" s="91"/>
-      <c r="B63" s="83"/>
-      <c r="C63" s="92"/>
-      <c r="D63" s="92"/>
-      <c r="E63" s="92"/>
-      <c r="F63" s="92"/>
-      <c r="G63" s="92"/>
-      <c r="H63" s="92"/>
-      <c r="I63" s="92"/>
-      <c r="J63" s="92"/>
-      <c r="K63" s="93"/>
-      <c r="L63" s="92"/>
-      <c r="M63" s="90"/>
+    <row r="63" spans="1:76" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="91" t="s">
+        <v>163</v>
+      </c>
+      <c r="B63" s="83">
+        <v>9501199250</v>
+      </c>
+      <c r="C63" s="98">
+        <v>46054</v>
+      </c>
+      <c r="D63" s="98">
+        <v>46418</v>
+      </c>
+      <c r="E63" s="92" t="s">
+        <v>139</v>
+      </c>
+      <c r="F63" s="92" t="s">
+        <v>164</v>
+      </c>
+      <c r="G63" s="92">
+        <v>41010100</v>
+      </c>
+      <c r="H63" s="92">
+        <v>7280</v>
+      </c>
+      <c r="I63" s="92" t="s">
+        <v>141</v>
+      </c>
+      <c r="J63" s="92">
+        <v>2662855</v>
+      </c>
+      <c r="K63" s="99">
+        <v>69429</v>
+      </c>
+      <c r="L63" s="102" t="s">
+        <v>211</v>
+      </c>
+      <c r="M63" s="103" t="s">
+        <v>166</v>
+      </c>
       <c r="N63" s="82"/>
       <c r="O63" s="83"/>
       <c r="P63" s="83"/>
@@ -9472,243 +9391,358 @@
       <c r="BW64" s="89"/>
       <c r="BX64" s="90"/>
     </row>
-    <row r="65" spans="1:139" s="9" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="66" t="s">
+    <row r="65" spans="1:139" x14ac:dyDescent="0.25">
+      <c r="A65" s="91"/>
+      <c r="B65" s="83"/>
+      <c r="C65" s="92"/>
+      <c r="D65" s="92"/>
+      <c r="E65" s="92"/>
+      <c r="F65" s="92"/>
+      <c r="G65" s="92"/>
+      <c r="H65" s="92"/>
+      <c r="I65" s="92"/>
+      <c r="J65" s="92"/>
+      <c r="K65" s="93"/>
+      <c r="L65" s="92"/>
+      <c r="M65" s="90"/>
+      <c r="N65" s="82"/>
+      <c r="O65" s="83"/>
+      <c r="P65" s="83"/>
+      <c r="Q65" s="84"/>
+      <c r="R65" s="84">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="S65" s="85"/>
+      <c r="T65" s="83"/>
+      <c r="U65" s="83"/>
+      <c r="V65" s="84"/>
+      <c r="W65" s="86">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
+      <c r="X65" s="87"/>
+      <c r="Y65" s="83"/>
+      <c r="Z65" s="83"/>
+      <c r="AA65" s="84"/>
+      <c r="AB65" s="86">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="AC65" s="87"/>
+      <c r="AD65" s="83"/>
+      <c r="AE65" s="83"/>
+      <c r="AF65" s="84"/>
+      <c r="AG65" s="86">
+        <f t="shared" si="27"/>
+        <v>0</v>
+      </c>
+      <c r="AH65" s="87"/>
+      <c r="AI65" s="83"/>
+      <c r="AJ65" s="83"/>
+      <c r="AK65" s="84"/>
+      <c r="AL65" s="86">
+        <f t="shared" si="28"/>
+        <v>0</v>
+      </c>
+      <c r="AM65" s="87"/>
+      <c r="AN65" s="83"/>
+      <c r="AO65" s="83"/>
+      <c r="AP65" s="84"/>
+      <c r="AQ65" s="86">
+        <f t="shared" si="29"/>
+        <v>0</v>
+      </c>
+      <c r="AR65" s="87"/>
+      <c r="AS65" s="83"/>
+      <c r="AT65" s="83"/>
+      <c r="AU65" s="84"/>
+      <c r="AV65" s="86">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="AW65" s="87"/>
+      <c r="AX65" s="83"/>
+      <c r="AY65" s="83"/>
+      <c r="AZ65" s="84"/>
+      <c r="BA65" s="86">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+      <c r="BB65" s="87"/>
+      <c r="BC65" s="83"/>
+      <c r="BD65" s="83"/>
+      <c r="BE65" s="84"/>
+      <c r="BF65" s="86">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="BG65" s="87"/>
+      <c r="BH65" s="83"/>
+      <c r="BI65" s="83"/>
+      <c r="BJ65" s="84"/>
+      <c r="BK65" s="86">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="BL65" s="87"/>
+      <c r="BM65" s="83"/>
+      <c r="BN65" s="83"/>
+      <c r="BO65" s="84"/>
+      <c r="BP65" s="86">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="BQ65" s="87"/>
+      <c r="BR65" s="83"/>
+      <c r="BS65" s="83"/>
+      <c r="BT65" s="84"/>
+      <c r="BU65" s="86">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="BV65" s="85">
+        <v>0</v>
+      </c>
+      <c r="BW65" s="89"/>
+      <c r="BX65" s="90"/>
+    </row>
+    <row r="66" spans="1:139" s="9" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="66" t="s">
         <v>95</v>
       </c>
-      <c r="B65" s="67"/>
-      <c r="C65" s="68"/>
-      <c r="D65" s="68"/>
-      <c r="E65" s="69"/>
-      <c r="F65" s="69"/>
-      <c r="G65" s="69"/>
-      <c r="H65" s="69"/>
-      <c r="I65" s="69"/>
-      <c r="J65" s="69"/>
-      <c r="K65" s="70"/>
-      <c r="L65" s="69"/>
-      <c r="M65" s="71"/>
-      <c r="N65" s="72"/>
-      <c r="O65" s="73"/>
-      <c r="P65" s="73"/>
-      <c r="Q65" s="74"/>
-      <c r="R65" s="74" t="str">
-        <f>IF(OR(P65="",Q65=""),"",P65-Q65)</f>
+      <c r="B66" s="67"/>
+      <c r="C66" s="68"/>
+      <c r="D66" s="68"/>
+      <c r="E66" s="69"/>
+      <c r="F66" s="69"/>
+      <c r="G66" s="69"/>
+      <c r="H66" s="69"/>
+      <c r="I66" s="69"/>
+      <c r="J66" s="69"/>
+      <c r="K66" s="70"/>
+      <c r="L66" s="69"/>
+      <c r="M66" s="71"/>
+      <c r="N66" s="72"/>
+      <c r="O66" s="73"/>
+      <c r="P66" s="73"/>
+      <c r="Q66" s="74"/>
+      <c r="R66" s="74" t="str">
+        <f>IF(OR(P66="",Q66=""),"",P66-Q66)</f>
         <v/>
       </c>
-      <c r="S65" s="75"/>
-      <c r="T65" s="73"/>
-      <c r="U65" s="73"/>
-      <c r="V65" s="74"/>
-      <c r="W65" s="76"/>
-      <c r="X65" s="77"/>
-      <c r="Y65" s="73"/>
-      <c r="Z65" s="73"/>
-      <c r="AA65" s="74"/>
-      <c r="AB65" s="76"/>
-      <c r="AC65" s="77"/>
-      <c r="AD65" s="73"/>
-      <c r="AE65" s="73"/>
-      <c r="AF65" s="74"/>
-      <c r="AG65" s="76" t="str">
-        <f t="shared" ref="AG65" si="36">IF(OR(AE65="",AF65=""),"",AE65-AF65)</f>
+      <c r="S66" s="75"/>
+      <c r="T66" s="73"/>
+      <c r="U66" s="73"/>
+      <c r="V66" s="74"/>
+      <c r="W66" s="76"/>
+      <c r="X66" s="77"/>
+      <c r="Y66" s="73"/>
+      <c r="Z66" s="73"/>
+      <c r="AA66" s="74"/>
+      <c r="AB66" s="76"/>
+      <c r="AC66" s="77"/>
+      <c r="AD66" s="73"/>
+      <c r="AE66" s="73"/>
+      <c r="AF66" s="74"/>
+      <c r="AG66" s="76" t="str">
+        <f t="shared" ref="AG66" si="36">IF(OR(AE66="",AF66=""),"",AE66-AF66)</f>
         <v/>
       </c>
-      <c r="AH65" s="77"/>
-      <c r="AI65" s="73"/>
-      <c r="AJ65" s="73"/>
-      <c r="AK65" s="74"/>
-      <c r="AL65" s="76" t="str">
-        <f t="shared" ref="AL65" si="37">IF(OR(AJ65="",AK65=""),"",AJ65-AK65)</f>
+      <c r="AH66" s="77"/>
+      <c r="AI66" s="73"/>
+      <c r="AJ66" s="73"/>
+      <c r="AK66" s="74"/>
+      <c r="AL66" s="76" t="str">
+        <f t="shared" ref="AL66" si="37">IF(OR(AJ66="",AK66=""),"",AJ66-AK66)</f>
         <v/>
       </c>
-      <c r="AM65" s="77"/>
-      <c r="AN65" s="73"/>
-      <c r="AO65" s="73"/>
-      <c r="AP65" s="74"/>
-      <c r="AQ65" s="76" t="str">
-        <f t="shared" ref="AQ65" si="38">IF(OR(AO65="",AP65=""),"",AO65-AP65)</f>
+      <c r="AM66" s="77"/>
+      <c r="AN66" s="73"/>
+      <c r="AO66" s="73"/>
+      <c r="AP66" s="74"/>
+      <c r="AQ66" s="76" t="str">
+        <f t="shared" ref="AQ66" si="38">IF(OR(AO66="",AP66=""),"",AO66-AP66)</f>
         <v/>
       </c>
-      <c r="AR65" s="77"/>
-      <c r="AS65" s="73"/>
-      <c r="AT65" s="73"/>
-      <c r="AU65" s="74"/>
-      <c r="AV65" s="76" t="str">
-        <f t="shared" ref="AV65" si="39">IF(OR(AT65="",AU65=""),"",AT65-AU65)</f>
+      <c r="AR66" s="77"/>
+      <c r="AS66" s="73"/>
+      <c r="AT66" s="73"/>
+      <c r="AU66" s="74"/>
+      <c r="AV66" s="76" t="str">
+        <f t="shared" ref="AV66" si="39">IF(OR(AT66="",AU66=""),"",AT66-AU66)</f>
         <v/>
       </c>
-      <c r="AW65" s="77"/>
-      <c r="AX65" s="73"/>
-      <c r="AY65" s="73"/>
-      <c r="AZ65" s="74"/>
-      <c r="BA65" s="76" t="str">
-        <f t="shared" ref="BA65" si="40">IF(OR(AY65="",AZ65=""),"",AY65-AZ65)</f>
+      <c r="AW66" s="77"/>
+      <c r="AX66" s="73"/>
+      <c r="AY66" s="73"/>
+      <c r="AZ66" s="74"/>
+      <c r="BA66" s="76" t="str">
+        <f t="shared" ref="BA66" si="40">IF(OR(AY66="",AZ66=""),"",AY66-AZ66)</f>
         <v/>
       </c>
-      <c r="BB65" s="77"/>
-      <c r="BC65" s="73"/>
-      <c r="BD65" s="73"/>
-      <c r="BE65" s="74"/>
-      <c r="BF65" s="76" t="str">
-        <f t="shared" ref="BF65" si="41">IF(OR(BD65="",BE65=""),"",BD65-BE65)</f>
+      <c r="BB66" s="77"/>
+      <c r="BC66" s="73"/>
+      <c r="BD66" s="73"/>
+      <c r="BE66" s="74"/>
+      <c r="BF66" s="76" t="str">
+        <f t="shared" ref="BF66" si="41">IF(OR(BD66="",BE66=""),"",BD66-BE66)</f>
         <v/>
       </c>
-      <c r="BG65" s="77"/>
-      <c r="BH65" s="73"/>
-      <c r="BI65" s="73"/>
-      <c r="BJ65" s="74"/>
-      <c r="BK65" s="76" t="str">
-        <f t="shared" ref="BK65" si="42">IF(OR(BI65="",BJ65=""),"",BI65-BJ65)</f>
+      <c r="BG66" s="77"/>
+      <c r="BH66" s="73"/>
+      <c r="BI66" s="73"/>
+      <c r="BJ66" s="74"/>
+      <c r="BK66" s="76" t="str">
+        <f t="shared" ref="BK66" si="42">IF(OR(BI66="",BJ66=""),"",BI66-BJ66)</f>
         <v/>
       </c>
-      <c r="BL65" s="77"/>
-      <c r="BM65" s="73"/>
-      <c r="BN65" s="73"/>
-      <c r="BO65" s="74"/>
-      <c r="BP65" s="76" t="str">
-        <f t="shared" ref="BP65" si="43">IF(OR(BN65="",BO65=""),"",BN65-BO65)</f>
+      <c r="BL66" s="77"/>
+      <c r="BM66" s="73"/>
+      <c r="BN66" s="73"/>
+      <c r="BO66" s="74"/>
+      <c r="BP66" s="76" t="str">
+        <f t="shared" ref="BP66" si="43">IF(OR(BN66="",BO66=""),"",BN66-BO66)</f>
         <v/>
       </c>
-      <c r="BQ65" s="77"/>
-      <c r="BR65" s="73"/>
-      <c r="BS65" s="73"/>
-      <c r="BT65" s="74"/>
-      <c r="BU65" s="76" t="str">
-        <f t="shared" ref="BU65" si="44">IF(OR(BS65="",BT65=""),"",BS65-BT65)</f>
+      <c r="BQ66" s="77"/>
+      <c r="BR66" s="73"/>
+      <c r="BS66" s="73"/>
+      <c r="BT66" s="74"/>
+      <c r="BU66" s="76" t="str">
+        <f t="shared" ref="BU66" si="44">IF(OR(BS66="",BT66=""),"",BS66-BT66)</f>
         <v/>
       </c>
-      <c r="BV65" s="75"/>
-      <c r="BW65" s="53"/>
-      <c r="BX65" s="49"/>
-      <c r="BY65"/>
-      <c r="BZ65"/>
-      <c r="CA65"/>
-      <c r="CB65"/>
-      <c r="CC65"/>
-      <c r="CD65"/>
-      <c r="CE65"/>
-      <c r="CF65"/>
-      <c r="CG65"/>
-      <c r="CH65"/>
-      <c r="CI65"/>
-      <c r="CJ65"/>
-      <c r="CK65"/>
-      <c r="CL65"/>
-      <c r="CM65"/>
-      <c r="CN65"/>
-      <c r="CO65"/>
-      <c r="CP65"/>
-      <c r="CQ65"/>
-      <c r="CR65"/>
-      <c r="CS65"/>
-      <c r="CT65"/>
-      <c r="CU65"/>
-      <c r="CV65"/>
-      <c r="CW65"/>
-      <c r="CX65"/>
-      <c r="CY65"/>
-      <c r="CZ65"/>
-      <c r="DA65"/>
-      <c r="DB65"/>
-      <c r="DC65"/>
-      <c r="DD65"/>
-      <c r="DE65"/>
-      <c r="DF65"/>
-      <c r="DG65"/>
-      <c r="DH65"/>
-      <c r="DI65"/>
-      <c r="DJ65"/>
-      <c r="DK65"/>
-      <c r="DL65"/>
-      <c r="DM65"/>
-      <c r="DN65"/>
-      <c r="DO65"/>
-      <c r="DP65"/>
-      <c r="DQ65"/>
-      <c r="DR65"/>
-      <c r="DS65"/>
-      <c r="DT65"/>
-      <c r="DU65"/>
-      <c r="DV65"/>
-      <c r="DW65"/>
-      <c r="DX65"/>
-      <c r="DY65"/>
-      <c r="DZ65"/>
-      <c r="EA65"/>
-      <c r="EB65"/>
-      <c r="EC65"/>
-      <c r="ED65"/>
-      <c r="EE65"/>
-      <c r="EF65"/>
-      <c r="EG65"/>
-      <c r="EH65"/>
-      <c r="EI65"/>
+      <c r="BV66" s="75"/>
+      <c r="BW66" s="53"/>
+      <c r="BX66" s="49"/>
+      <c r="BY66"/>
+      <c r="BZ66"/>
+      <c r="CA66"/>
+      <c r="CB66"/>
+      <c r="CC66"/>
+      <c r="CD66"/>
+      <c r="CE66"/>
+      <c r="CF66"/>
+      <c r="CG66"/>
+      <c r="CH66"/>
+      <c r="CI66"/>
+      <c r="CJ66"/>
+      <c r="CK66"/>
+      <c r="CL66"/>
+      <c r="CM66"/>
+      <c r="CN66"/>
+      <c r="CO66"/>
+      <c r="CP66"/>
+      <c r="CQ66"/>
+      <c r="CR66"/>
+      <c r="CS66"/>
+      <c r="CT66"/>
+      <c r="CU66"/>
+      <c r="CV66"/>
+      <c r="CW66"/>
+      <c r="CX66"/>
+      <c r="CY66"/>
+      <c r="CZ66"/>
+      <c r="DA66"/>
+      <c r="DB66"/>
+      <c r="DC66"/>
+      <c r="DD66"/>
+      <c r="DE66"/>
+      <c r="DF66"/>
+      <c r="DG66"/>
+      <c r="DH66"/>
+      <c r="DI66"/>
+      <c r="DJ66"/>
+      <c r="DK66"/>
+      <c r="DL66"/>
+      <c r="DM66"/>
+      <c r="DN66"/>
+      <c r="DO66"/>
+      <c r="DP66"/>
+      <c r="DQ66"/>
+      <c r="DR66"/>
+      <c r="DS66"/>
+      <c r="DT66"/>
+      <c r="DU66"/>
+      <c r="DV66"/>
+      <c r="DW66"/>
+      <c r="DX66"/>
+      <c r="DY66"/>
+      <c r="DZ66"/>
+      <c r="EA66"/>
+      <c r="EB66"/>
+      <c r="EC66"/>
+      <c r="ED66"/>
+      <c r="EE66"/>
+      <c r="EF66"/>
+      <c r="EG66"/>
+      <c r="EH66"/>
+      <c r="EI66"/>
     </row>
-    <row r="66" spans="1:139" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="67" spans="1:139" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>96</v>
       </c>
-      <c r="AA66" s="3"/>
-      <c r="BV66" s="95"/>
+      <c r="AA67" s="3"/>
+      <c r="BV67" s="95"/>
     </row>
   </sheetData>
-  <autoFilter ref="A14:BY18" xr:uid="{177F1DEB-197D-49C6-A2E3-152C1AC7B373}"/>
-  <mergeCells count="40">
-    <mergeCell ref="BQ11:BU11"/>
+  <autoFilter ref="A15:BY19" xr:uid="{177F1DEB-197D-49C6-A2E3-152C1AC7B373}"/>
+  <mergeCells count="39">
     <mergeCell ref="BQ13:BU13"/>
-    <mergeCell ref="S11:W11"/>
-    <mergeCell ref="N11:R11"/>
-    <mergeCell ref="X11:AB11"/>
-    <mergeCell ref="AC11:AG11"/>
-    <mergeCell ref="AH11:AL11"/>
-    <mergeCell ref="AM11:AQ11"/>
-    <mergeCell ref="AR11:AV11"/>
-    <mergeCell ref="AW11:BA11"/>
-    <mergeCell ref="BB11:BF11"/>
-    <mergeCell ref="BG11:BK11"/>
-    <mergeCell ref="BL11:BP11"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="BB14:BF14"/>
+    <mergeCell ref="BG14:BK14"/>
+    <mergeCell ref="BL14:BP14"/>
+    <mergeCell ref="N13:R13"/>
     <mergeCell ref="S13:W13"/>
-    <mergeCell ref="N13:R13"/>
     <mergeCell ref="X13:AB13"/>
-    <mergeCell ref="BB12:BF12"/>
-    <mergeCell ref="BG12:BK12"/>
-    <mergeCell ref="BL12:BP12"/>
     <mergeCell ref="AC13:AG13"/>
     <mergeCell ref="AH13:AL13"/>
     <mergeCell ref="AM13:AQ13"/>
     <mergeCell ref="AR13:AV13"/>
     <mergeCell ref="AW13:BA13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="BQ12:BU12"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="L13:M13"/>
     <mergeCell ref="BB13:BF13"/>
     <mergeCell ref="BG13:BK13"/>
     <mergeCell ref="BL13:BP13"/>
+    <mergeCell ref="AC14:AG14"/>
+    <mergeCell ref="AH14:AL14"/>
+    <mergeCell ref="AM14:AQ14"/>
+    <mergeCell ref="AR14:AV14"/>
+    <mergeCell ref="AW14:BA14"/>
+    <mergeCell ref="BQ12:BU12"/>
+    <mergeCell ref="BQ14:BU14"/>
+    <mergeCell ref="S12:W12"/>
     <mergeCell ref="N12:R12"/>
-    <mergeCell ref="S12:W12"/>
     <mergeCell ref="X12:AB12"/>
     <mergeCell ref="AC12:AG12"/>
     <mergeCell ref="AH12:AL12"/>
     <mergeCell ref="AM12:AQ12"/>
     <mergeCell ref="AR12:AV12"/>
     <mergeCell ref="AW12:BA12"/>
+    <mergeCell ref="BB12:BF12"/>
+    <mergeCell ref="BG12:BK12"/>
+    <mergeCell ref="BL12:BP12"/>
+    <mergeCell ref="S14:W14"/>
+    <mergeCell ref="N14:R14"/>
+    <mergeCell ref="X14:AB14"/>
   </mergeCells>
-  <conditionalFormatting sqref="Q65 V65 AA65 AF65 AK65 AP65 AU65 AZ65 BE65 BJ65 BO65 BT65">
-    <cfRule type="expression" dxfId="2" priority="8">
-      <formula>IF(AND(P65&gt;0,Q65=0),TRUE,FALSE)</formula>
+  <conditionalFormatting sqref="Q66 V66 AA66 AF66 AK66 AP66 AU66 AZ66 BE66 BJ66 BO66 BT66">
+    <cfRule type="expression" dxfId="6" priority="8">
+      <formula>IF(AND(P66&gt;0,Q66=0),TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BT10 V65:X65 AB65:AC65 AG65:AH65 AL65:AM65 AQ65:AR65 AV65:AW65 BA65:BB65 BF65:BG65 BK65:BL65 BP65:BQ65 BU65">
-    <cfRule type="expression" dxfId="1" priority="9">
-      <formula>IF(AND(U10&lt;&gt;"",V10="",TODAY()&gt;DATE(YEAR(TODAY()),MONTH(DATEVALUE("1-"&amp;LEFT(#REF!,3)&amp;"-1900")),20)),TRUE,FALSE)</formula>
+  <conditionalFormatting sqref="BT11 V66:X66 AB66:AC66 AG66:AH66 AL66:AM66 AQ66:AR66 AV66:AW66 BA66:BB66 BF66:BG66 BK66:BL66 BP66:BQ66 BU66">
+    <cfRule type="expression" dxfId="5" priority="9">
+      <formula>IF(AND(U11&lt;&gt;"",V11="",TODAY()&gt;DATE(YEAR(TODAY()),MONTH(DATEVALUE("1-"&amp;LEFT(#REF!,3)&amp;"-1900")),20)),TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BW11:BW12">
-    <cfRule type="expression" dxfId="0" priority="7">
-      <formula>IF(BW11&lt;0,TRUE,FALSE)</formula>
+  <conditionalFormatting sqref="BW12:BW13">
+    <cfRule type="expression" dxfId="4" priority="7">
+      <formula>IF(BW12&lt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9717,26 +9751,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19b1ad6d-7bbd-4338-adb0-a51e11e836c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002B3B1E9AF76D8540A21B723585178CF2" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9038a3d09b9201f70a536d69b3ffdde9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="19b1ad6d-7bbd-4338-adb0-a51e11e836c7" xmlns:ns3="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c9f1b7b0d1eaccac7f713200a7ec3f32" ns2:_="" ns3:_="">
     <xsd:import namespace="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
@@ -9979,26 +9993,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09"/>
-    <ds:schemaRef ds:uri="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="19b1ad6d-7bbd-4338-adb0-a51e11e836c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0B6774AE-0D33-4944-9922-507715E1B0E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10015,4 +10030,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3614A8F8-9AED-4C02-B640-81A3A1FEB080}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC2B212-31BA-49FB-B215-9E14B2C60948}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8aede0e7-b4a5-4e74-9fbf-51d976a6ba09"/>
+    <ds:schemaRef ds:uri="19b1ad6d-7bbd-4338-adb0-a51e11e836c7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>